<commit_message>
/contact: "form below" links to the form; forms get their sheet's name as id
The source links "form below" to #contact, which no element there has. The
importer now keeps the link as #contact-form, and form-minimal-light gives
each form its sheet's name as its id (contact-form, fraud-form,
news-alert-form) unless the page already uses it.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-contact.report.xlsx
+++ b/tools/importer/reports/import-contact.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1275" uniqueCount="673">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1286" uniqueCount="678">
   <si>
     <t>_reportFile</t>
   </si>
@@ -73,6 +73,27 @@
     <t>https://www.highmark.com/because-life</t>
   </si>
   <si>
+    <t>contact-thank-you.report.json</t>
+  </si>
+  <si>
+    <t>[]</t>
+  </si>
+  <si>
+    <t>contact-thank-you</t>
+  </si>
+  <si>
+    <t>fraud-thank-you</t>
+  </si>
+  <si>
+    <t>2026-10-14T08:30:39.378Z</t>
+  </si>
+  <si>
+    <t>Thank You</t>
+  </si>
+  <si>
+    <t>https://www.highmark.com/contact-thank-you</t>
+  </si>
+  <si>
     <t>contact.report.json</t>
   </si>
   <si>
@@ -82,7 +103,7 @@
     <t>contact</t>
   </si>
   <si>
-    <t>2026-10-14T08:30:32.469Z</t>
+    <t>2026-10-14T09:06:59.963Z</t>
   </si>
   <si>
     <t>Contact Highmark</t>
@@ -113,12 +134,6 @@
   </si>
   <si>
     <t>fraud-thank-you.report.json</t>
-  </si>
-  <si>
-    <t>[]</t>
-  </si>
-  <si>
-    <t>fraud-thank-you</t>
   </si>
   <si>
     <t>2026-10-14T07:13:24.168Z</t>
@@ -2418,7 +2433,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K116"/>
+  <dimension ref="A1:K117"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="50" customWidth="1"/>
@@ -2523,24 +2538,24 @@
         <v>15</v>
       </c>
       <c r="H3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C4" t="s">
         <v>13</v>
@@ -2552,7 +2567,7 @@
         <v>13</v>
       </c>
       <c r="F4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G4" t="s">
         <v>15</v>
@@ -2593,24 +2608,24 @@
         <v>15</v>
       </c>
       <c r="H5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="I5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="J5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="K5" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B6" t="s">
-        <v>40</v>
+        <v>21</v>
       </c>
       <c r="C6" t="s">
         <v>13</v>
@@ -2622,112 +2637,112 @@
         <v>13</v>
       </c>
       <c r="F6" t="s">
+        <v>23</v>
+      </c>
+      <c r="G6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I6" t="s">
         <v>41</v>
       </c>
-      <c r="G6" t="s">
-        <v>15</v>
-      </c>
-      <c r="H6" t="s">
+      <c r="J6" t="s">
         <v>42</v>
       </c>
-      <c r="I6" t="s">
+      <c r="K6" t="s">
         <v>43</v>
-      </c>
-      <c r="J6" t="s">
-        <v>44</v>
-      </c>
-      <c r="K6" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>44</v>
+      </c>
+      <c r="B7" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" t="s">
         <v>46</v>
       </c>
-      <c r="B7" t="s">
+      <c r="G7" t="s">
+        <v>15</v>
+      </c>
+      <c r="H7" t="s">
         <v>47</v>
       </c>
-      <c r="C7" t="s">
-        <v>13</v>
-      </c>
-      <c r="D7" t="s">
-        <v>13</v>
-      </c>
-      <c r="E7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F7" t="s">
+      <c r="I7" t="s">
         <v>48</v>
       </c>
-      <c r="G7" t="s">
-        <v>15</v>
-      </c>
-      <c r="H7" t="s">
-        <v>16</v>
-      </c>
-      <c r="I7" t="s">
+      <c r="J7" t="s">
         <v>49</v>
       </c>
-      <c r="J7" t="s">
+      <c r="K7" t="s">
         <v>50</v>
-      </c>
-      <c r="K7" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B8" t="s">
         <v>52</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" t="s">
         <v>53</v>
       </c>
-      <c r="C8" t="s">
-        <v>13</v>
-      </c>
-      <c r="D8" t="s">
-        <v>13</v>
-      </c>
-      <c r="E8" t="s">
-        <v>13</v>
-      </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
+        <v>15</v>
+      </c>
+      <c r="H8" t="s">
+        <v>16</v>
+      </c>
+      <c r="I8" t="s">
         <v>54</v>
       </c>
-      <c r="G8" t="s">
-        <v>15</v>
-      </c>
-      <c r="H8" t="s">
+      <c r="J8" t="s">
         <v>55</v>
       </c>
-      <c r="I8" t="s">
+      <c r="K8" t="s">
         <v>56</v>
-      </c>
-      <c r="J8" t="s">
-        <v>57</v>
-      </c>
-      <c r="K8" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>57</v>
+      </c>
+      <c r="B9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F9" t="s">
         <v>59</v>
-      </c>
-      <c r="B9" t="s">
-        <v>34</v>
-      </c>
-      <c r="C9" t="s">
-        <v>13</v>
-      </c>
-      <c r="D9" t="s">
-        <v>13</v>
-      </c>
-      <c r="E9" t="s">
-        <v>13</v>
-      </c>
-      <c r="F9" t="s">
-        <v>60</v>
       </c>
       <c r="G9" t="s">
         <v>15</v>
@@ -2750,7 +2765,7 @@
         <v>64</v>
       </c>
       <c r="B10" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="C10" t="s">
         <v>13</v>
@@ -2774,18 +2789,18 @@
         <v>66</v>
       </c>
       <c r="J10" t="s">
-        <v>13</v>
+        <v>67</v>
       </c>
       <c r="K10" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B11" t="s">
-        <v>69</v>
+        <v>21</v>
       </c>
       <c r="C11" t="s">
         <v>13</v>
@@ -2803,42 +2818,42 @@
         <v>15</v>
       </c>
       <c r="H11" t="s">
+        <v>70</v>
+      </c>
+      <c r="I11" t="s">
         <v>71</v>
       </c>
-      <c r="I11" t="s">
+      <c r="J11" t="s">
+        <v>13</v>
+      </c>
+      <c r="K11" t="s">
         <v>72</v>
-      </c>
-      <c r="J11" t="s">
-        <v>73</v>
-      </c>
-      <c r="K11" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>73</v>
+      </c>
+      <c r="B12" t="s">
+        <v>74</v>
+      </c>
+      <c r="C12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D12" t="s">
+        <v>13</v>
+      </c>
+      <c r="E12" t="s">
+        <v>13</v>
+      </c>
+      <c r="F12" t="s">
         <v>75</v>
       </c>
-      <c r="B12" t="s">
-        <v>34</v>
-      </c>
-      <c r="C12" t="s">
-        <v>13</v>
-      </c>
-      <c r="D12" t="s">
-        <v>13</v>
-      </c>
-      <c r="E12" t="s">
-        <v>13</v>
-      </c>
-      <c r="F12" t="s">
+      <c r="G12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H12" t="s">
         <v>76</v>
-      </c>
-      <c r="G12" t="s">
-        <v>15</v>
-      </c>
-      <c r="H12" t="s">
-        <v>71</v>
       </c>
       <c r="I12" t="s">
         <v>77</v>
@@ -2855,7 +2870,7 @@
         <v>80</v>
       </c>
       <c r="B13" t="s">
-        <v>47</v>
+        <v>21</v>
       </c>
       <c r="C13" t="s">
         <v>13</v>
@@ -2873,118 +2888,118 @@
         <v>15</v>
       </c>
       <c r="H13" t="s">
+        <v>76</v>
+      </c>
+      <c r="I13" t="s">
         <v>82</v>
       </c>
-      <c r="I13" t="s">
+      <c r="J13" t="s">
         <v>83</v>
       </c>
-      <c r="J13" t="s">
+      <c r="K13" t="s">
         <v>84</v>
-      </c>
-      <c r="K13" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>85</v>
+      </c>
+      <c r="B14" t="s">
+        <v>52</v>
+      </c>
+      <c r="C14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D14" t="s">
+        <v>13</v>
+      </c>
+      <c r="E14" t="s">
+        <v>13</v>
+      </c>
+      <c r="F14" t="s">
         <v>86</v>
       </c>
-      <c r="B14" t="s">
+      <c r="G14" t="s">
+        <v>15</v>
+      </c>
+      <c r="H14" t="s">
         <v>87</v>
       </c>
-      <c r="C14" t="s">
-        <v>13</v>
-      </c>
-      <c r="D14" t="s">
-        <v>13</v>
-      </c>
-      <c r="E14" t="s">
-        <v>13</v>
-      </c>
-      <c r="F14" t="s">
+      <c r="I14" t="s">
         <v>88</v>
       </c>
-      <c r="G14" t="s">
-        <v>15</v>
-      </c>
-      <c r="H14" t="s">
-        <v>16</v>
-      </c>
-      <c r="I14" t="s">
+      <c r="J14" t="s">
         <v>89</v>
       </c>
-      <c r="J14" t="s">
+      <c r="K14" t="s">
         <v>90</v>
-      </c>
-      <c r="K14" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>91</v>
+      </c>
+      <c r="B15" t="s">
         <v>92</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
+        <v>13</v>
+      </c>
+      <c r="D15" t="s">
+        <v>13</v>
+      </c>
+      <c r="E15" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15" t="s">
         <v>93</v>
       </c>
-      <c r="C15" t="s">
-        <v>13</v>
-      </c>
-      <c r="D15" t="s">
-        <v>13</v>
-      </c>
-      <c r="E15" t="s">
-        <v>13</v>
-      </c>
-      <c r="F15" t="s">
+      <c r="G15" t="s">
+        <v>15</v>
+      </c>
+      <c r="H15" t="s">
+        <v>16</v>
+      </c>
+      <c r="I15" t="s">
         <v>94</v>
       </c>
-      <c r="G15" t="s">
-        <v>15</v>
-      </c>
-      <c r="H15" t="s">
-        <v>42</v>
-      </c>
-      <c r="I15" t="s">
+      <c r="J15" t="s">
         <v>95</v>
       </c>
-      <c r="J15" t="s">
+      <c r="K15" t="s">
         <v>96</v>
-      </c>
-      <c r="K15" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>97</v>
+      </c>
+      <c r="B16" t="s">
         <v>98</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
+        <v>13</v>
+      </c>
+      <c r="D16" t="s">
+        <v>13</v>
+      </c>
+      <c r="E16" t="s">
+        <v>13</v>
+      </c>
+      <c r="F16" t="s">
         <v>99</v>
       </c>
-      <c r="C16" t="s">
-        <v>13</v>
-      </c>
-      <c r="D16" t="s">
-        <v>13</v>
-      </c>
-      <c r="E16" t="s">
-        <v>13</v>
-      </c>
-      <c r="F16" t="s">
+      <c r="G16" t="s">
+        <v>15</v>
+      </c>
+      <c r="H16" t="s">
+        <v>47</v>
+      </c>
+      <c r="I16" t="s">
         <v>100</v>
       </c>
-      <c r="G16" t="s">
-        <v>15</v>
-      </c>
-      <c r="H16" t="s">
-        <v>100</v>
-      </c>
-      <c r="I16" t="s">
+      <c r="J16" t="s">
         <v>101</v>
-      </c>
-      <c r="J16" t="s">
-        <v>13</v>
       </c>
       <c r="K16" t="s">
         <v>102</v>
@@ -3013,77 +3028,77 @@
         <v>15</v>
       </c>
       <c r="H17" t="s">
+        <v>105</v>
+      </c>
+      <c r="I17" t="s">
         <v>106</v>
       </c>
-      <c r="I17" t="s">
+      <c r="J17" t="s">
+        <v>13</v>
+      </c>
+      <c r="K17" t="s">
         <v>107</v>
-      </c>
-      <c r="J17" t="s">
-        <v>108</v>
-      </c>
-      <c r="K17" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>108</v>
+      </c>
+      <c r="B18" t="s">
+        <v>109</v>
+      </c>
+      <c r="C18" t="s">
+        <v>13</v>
+      </c>
+      <c r="D18" t="s">
+        <v>13</v>
+      </c>
+      <c r="E18" t="s">
+        <v>13</v>
+      </c>
+      <c r="F18" t="s">
         <v>110</v>
       </c>
-      <c r="B18" t="s">
+      <c r="G18" t="s">
+        <v>15</v>
+      </c>
+      <c r="H18" t="s">
         <v>111</v>
       </c>
-      <c r="C18" t="s">
-        <v>13</v>
-      </c>
-      <c r="D18" t="s">
-        <v>13</v>
-      </c>
-      <c r="E18" t="s">
-        <v>13</v>
-      </c>
-      <c r="F18" t="s">
+      <c r="I18" t="s">
         <v>112</v>
       </c>
-      <c r="G18" t="s">
-        <v>15</v>
-      </c>
-      <c r="H18" t="s">
+      <c r="J18" t="s">
         <v>113</v>
       </c>
-      <c r="I18" t="s">
+      <c r="K18" t="s">
         <v>114</v>
-      </c>
-      <c r="J18" t="s">
-        <v>115</v>
-      </c>
-      <c r="K18" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>115</v>
+      </c>
+      <c r="B19" t="s">
+        <v>116</v>
+      </c>
+      <c r="C19" t="s">
+        <v>13</v>
+      </c>
+      <c r="D19" t="s">
+        <v>13</v>
+      </c>
+      <c r="E19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F19" t="s">
         <v>117</v>
       </c>
-      <c r="B19" t="s">
-        <v>104</v>
-      </c>
-      <c r="C19" t="s">
-        <v>13</v>
-      </c>
-      <c r="D19" t="s">
-        <v>13</v>
-      </c>
-      <c r="E19" t="s">
-        <v>13</v>
-      </c>
-      <c r="F19" t="s">
+      <c r="G19" t="s">
+        <v>15</v>
+      </c>
+      <c r="H19" t="s">
         <v>118</v>
-      </c>
-      <c r="G19" t="s">
-        <v>15</v>
-      </c>
-      <c r="H19" t="s">
-        <v>106</v>
       </c>
       <c r="I19" t="s">
         <v>119</v>
@@ -3100,270 +3115,270 @@
         <v>122</v>
       </c>
       <c r="B20" t="s">
+        <v>109</v>
+      </c>
+      <c r="C20" t="s">
+        <v>13</v>
+      </c>
+      <c r="D20" t="s">
+        <v>13</v>
+      </c>
+      <c r="E20" t="s">
+        <v>13</v>
+      </c>
+      <c r="F20" t="s">
         <v>123</v>
       </c>
-      <c r="C20" t="s">
-        <v>13</v>
-      </c>
-      <c r="D20" t="s">
-        <v>13</v>
-      </c>
-      <c r="E20" t="s">
-        <v>13</v>
-      </c>
-      <c r="F20" t="s">
+      <c r="G20" t="s">
+        <v>15</v>
+      </c>
+      <c r="H20" t="s">
+        <v>111</v>
+      </c>
+      <c r="I20" t="s">
         <v>124</v>
       </c>
-      <c r="G20" t="s">
-        <v>15</v>
-      </c>
-      <c r="H20" t="s">
-        <v>16</v>
-      </c>
-      <c r="I20" t="s">
+      <c r="J20" t="s">
         <v>125</v>
       </c>
-      <c r="J20" t="s">
+      <c r="K20" t="s">
         <v>126</v>
-      </c>
-      <c r="K20" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>127</v>
+      </c>
+      <c r="B21" t="s">
         <v>128</v>
       </c>
-      <c r="B21" t="s">
+      <c r="C21" t="s">
+        <v>13</v>
+      </c>
+      <c r="D21" t="s">
+        <v>13</v>
+      </c>
+      <c r="E21" t="s">
+        <v>13</v>
+      </c>
+      <c r="F21" t="s">
         <v>129</v>
       </c>
-      <c r="C21" t="s">
-        <v>13</v>
-      </c>
-      <c r="D21" t="s">
-        <v>13</v>
-      </c>
-      <c r="E21" t="s">
-        <v>13</v>
-      </c>
-      <c r="F21" t="s">
+      <c r="G21" t="s">
+        <v>15</v>
+      </c>
+      <c r="H21" t="s">
+        <v>16</v>
+      </c>
+      <c r="I21" t="s">
         <v>130</v>
       </c>
-      <c r="G21" t="s">
-        <v>15</v>
-      </c>
-      <c r="H21" t="s">
+      <c r="J21" t="s">
         <v>131</v>
       </c>
-      <c r="I21" t="s">
+      <c r="K21" t="s">
         <v>132</v>
-      </c>
-      <c r="J21" t="s">
-        <v>133</v>
-      </c>
-      <c r="K21" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>133</v>
+      </c>
+      <c r="B22" t="s">
+        <v>134</v>
+      </c>
+      <c r="C22" t="s">
+        <v>13</v>
+      </c>
+      <c r="D22" t="s">
+        <v>13</v>
+      </c>
+      <c r="E22" t="s">
+        <v>13</v>
+      </c>
+      <c r="F22" t="s">
         <v>135</v>
       </c>
-      <c r="B22" t="s">
+      <c r="G22" t="s">
+        <v>15</v>
+      </c>
+      <c r="H22" t="s">
         <v>136</v>
       </c>
-      <c r="C22" t="s">
-        <v>13</v>
-      </c>
-      <c r="D22" t="s">
-        <v>13</v>
-      </c>
-      <c r="E22" t="s">
-        <v>13</v>
-      </c>
-      <c r="F22" t="s">
+      <c r="I22" t="s">
         <v>137</v>
       </c>
-      <c r="G22" t="s">
-        <v>15</v>
-      </c>
-      <c r="H22" t="s">
-        <v>131</v>
-      </c>
-      <c r="I22" t="s">
+      <c r="J22" t="s">
         <v>138</v>
       </c>
-      <c r="J22" t="s">
+      <c r="K22" t="s">
         <v>139</v>
-      </c>
-      <c r="K22" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>140</v>
+      </c>
+      <c r="B23" t="s">
         <v>141</v>
       </c>
-      <c r="B23" t="s">
+      <c r="C23" t="s">
+        <v>13</v>
+      </c>
+      <c r="D23" t="s">
+        <v>13</v>
+      </c>
+      <c r="E23" t="s">
+        <v>13</v>
+      </c>
+      <c r="F23" t="s">
         <v>142</v>
       </c>
-      <c r="C23" t="s">
-        <v>13</v>
-      </c>
-      <c r="D23" t="s">
-        <v>13</v>
-      </c>
-      <c r="E23" t="s">
-        <v>13</v>
-      </c>
-      <c r="F23" t="s">
+      <c r="G23" t="s">
+        <v>15</v>
+      </c>
+      <c r="H23" t="s">
+        <v>136</v>
+      </c>
+      <c r="I23" t="s">
         <v>143</v>
       </c>
-      <c r="G23" t="s">
-        <v>15</v>
-      </c>
-      <c r="H23" t="s">
-        <v>131</v>
-      </c>
-      <c r="I23" t="s">
+      <c r="J23" t="s">
         <v>144</v>
       </c>
-      <c r="J23" t="s">
+      <c r="K23" t="s">
         <v>145</v>
-      </c>
-      <c r="K23" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>146</v>
+      </c>
+      <c r="B24" t="s">
         <v>147</v>
       </c>
-      <c r="B24" t="s">
+      <c r="C24" t="s">
+        <v>13</v>
+      </c>
+      <c r="D24" t="s">
+        <v>13</v>
+      </c>
+      <c r="E24" t="s">
+        <v>13</v>
+      </c>
+      <c r="F24" t="s">
         <v>148</v>
       </c>
-      <c r="C24" t="s">
-        <v>13</v>
-      </c>
-      <c r="D24" t="s">
-        <v>13</v>
-      </c>
-      <c r="E24" t="s">
-        <v>13</v>
-      </c>
-      <c r="F24" t="s">
+      <c r="G24" t="s">
+        <v>15</v>
+      </c>
+      <c r="H24" t="s">
+        <v>136</v>
+      </c>
+      <c r="I24" t="s">
         <v>149</v>
       </c>
-      <c r="G24" t="s">
-        <v>15</v>
-      </c>
-      <c r="H24" t="s">
-        <v>131</v>
-      </c>
-      <c r="I24" t="s">
+      <c r="J24" t="s">
         <v>150</v>
       </c>
-      <c r="J24" t="s">
+      <c r="K24" t="s">
         <v>151</v>
-      </c>
-      <c r="K24" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>152</v>
+      </c>
+      <c r="B25" t="s">
         <v>153</v>
       </c>
-      <c r="B25" t="s">
+      <c r="C25" t="s">
+        <v>13</v>
+      </c>
+      <c r="D25" t="s">
+        <v>13</v>
+      </c>
+      <c r="E25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F25" t="s">
         <v>154</v>
       </c>
-      <c r="C25" t="s">
-        <v>13</v>
-      </c>
-      <c r="D25" t="s">
-        <v>13</v>
-      </c>
-      <c r="E25" t="s">
-        <v>13</v>
-      </c>
-      <c r="F25" t="s">
+      <c r="G25" t="s">
+        <v>15</v>
+      </c>
+      <c r="H25" t="s">
+        <v>136</v>
+      </c>
+      <c r="I25" t="s">
         <v>155</v>
       </c>
-      <c r="G25" t="s">
-        <v>15</v>
-      </c>
-      <c r="H25" t="s">
-        <v>131</v>
-      </c>
-      <c r="I25" t="s">
+      <c r="J25" t="s">
         <v>156</v>
       </c>
-      <c r="J25" t="s">
+      <c r="K25" t="s">
         <v>157</v>
-      </c>
-      <c r="K25" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>158</v>
+      </c>
+      <c r="B26" t="s">
         <v>159</v>
       </c>
-      <c r="B26" t="s">
+      <c r="C26" t="s">
+        <v>13</v>
+      </c>
+      <c r="D26" t="s">
+        <v>13</v>
+      </c>
+      <c r="E26" t="s">
+        <v>13</v>
+      </c>
+      <c r="F26" t="s">
         <v>160</v>
       </c>
-      <c r="C26" t="s">
-        <v>13</v>
-      </c>
-      <c r="D26" t="s">
-        <v>13</v>
-      </c>
-      <c r="E26" t="s">
-        <v>13</v>
-      </c>
-      <c r="F26" t="s">
+      <c r="G26" t="s">
+        <v>15</v>
+      </c>
+      <c r="H26" t="s">
+        <v>136</v>
+      </c>
+      <c r="I26" t="s">
         <v>161</v>
       </c>
-      <c r="G26" t="s">
-        <v>15</v>
-      </c>
-      <c r="H26" t="s">
+      <c r="J26" t="s">
         <v>162</v>
       </c>
-      <c r="I26" t="s">
+      <c r="K26" t="s">
         <v>163</v>
-      </c>
-      <c r="J26" t="s">
-        <v>164</v>
-      </c>
-      <c r="K26" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>164</v>
+      </c>
+      <c r="B27" t="s">
+        <v>165</v>
+      </c>
+      <c r="C27" t="s">
+        <v>13</v>
+      </c>
+      <c r="D27" t="s">
+        <v>13</v>
+      </c>
+      <c r="E27" t="s">
+        <v>13</v>
+      </c>
+      <c r="F27" t="s">
         <v>166</v>
       </c>
-      <c r="B27" t="s">
-        <v>13</v>
-      </c>
-      <c r="C27" t="s">
-        <v>13</v>
-      </c>
-      <c r="D27">
-        <v>2</v>
-      </c>
-      <c r="E27" t="s">
-        <v>13</v>
-      </c>
-      <c r="F27" t="s">
+      <c r="G27" t="s">
+        <v>15</v>
+      </c>
+      <c r="H27" t="s">
         <v>167</v>
-      </c>
-      <c r="G27" t="s">
-        <v>15</v>
-      </c>
-      <c r="H27" t="s">
-        <v>13</v>
       </c>
       <c r="I27" t="s">
         <v>168</v>
@@ -3380,101 +3395,101 @@
         <v>171</v>
       </c>
       <c r="B28" t="s">
+        <v>13</v>
+      </c>
+      <c r="C28" t="s">
+        <v>13</v>
+      </c>
+      <c r="D28">
+        <v>2</v>
+      </c>
+      <c r="E28" t="s">
+        <v>13</v>
+      </c>
+      <c r="F28" t="s">
         <v>172</v>
       </c>
-      <c r="C28" t="s">
-        <v>13</v>
-      </c>
-      <c r="D28" t="s">
-        <v>13</v>
-      </c>
-      <c r="E28" t="s">
-        <v>13</v>
-      </c>
-      <c r="F28" t="s">
+      <c r="G28" t="s">
+        <v>15</v>
+      </c>
+      <c r="H28" t="s">
+        <v>13</v>
+      </c>
+      <c r="I28" t="s">
         <v>173</v>
       </c>
-      <c r="G28" t="s">
-        <v>15</v>
-      </c>
-      <c r="H28" t="s">
+      <c r="J28" t="s">
         <v>174</v>
       </c>
-      <c r="I28" t="s">
+      <c r="K28" t="s">
         <v>175</v>
-      </c>
-      <c r="J28" t="s">
-        <v>176</v>
-      </c>
-      <c r="K28" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>176</v>
+      </c>
+      <c r="B29" t="s">
+        <v>177</v>
+      </c>
+      <c r="C29" t="s">
+        <v>13</v>
+      </c>
+      <c r="D29" t="s">
+        <v>13</v>
+      </c>
+      <c r="E29" t="s">
+        <v>13</v>
+      </c>
+      <c r="F29" t="s">
         <v>178</v>
       </c>
-      <c r="B29" t="s">
-        <v>21</v>
-      </c>
-      <c r="C29" t="s">
-        <v>13</v>
-      </c>
-      <c r="D29" t="s">
-        <v>13</v>
-      </c>
-      <c r="E29" t="s">
-        <v>13</v>
-      </c>
-      <c r="F29" t="s">
+      <c r="G29" t="s">
+        <v>15</v>
+      </c>
+      <c r="H29" t="s">
         <v>179</v>
       </c>
-      <c r="G29" t="s">
-        <v>15</v>
-      </c>
-      <c r="H29" t="s">
+      <c r="I29" t="s">
         <v>180</v>
       </c>
-      <c r="I29" t="s">
+      <c r="J29" t="s">
         <v>181</v>
       </c>
-      <c r="J29" t="s">
+      <c r="K29" t="s">
         <v>182</v>
-      </c>
-      <c r="K29" t="s">
-        <v>183</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>183</v>
+      </c>
+      <c r="B30" t="s">
+        <v>28</v>
+      </c>
+      <c r="C30" t="s">
+        <v>13</v>
+      </c>
+      <c r="D30" t="s">
+        <v>13</v>
+      </c>
+      <c r="E30" t="s">
+        <v>13</v>
+      </c>
+      <c r="F30" t="s">
         <v>184</v>
       </c>
-      <c r="B30" t="s">
-        <v>111</v>
-      </c>
-      <c r="C30" t="s">
-        <v>13</v>
-      </c>
-      <c r="D30" t="s">
-        <v>13</v>
-      </c>
-      <c r="E30" t="s">
-        <v>13</v>
-      </c>
-      <c r="F30" t="s">
+      <c r="G30" t="s">
+        <v>15</v>
+      </c>
+      <c r="H30" t="s">
         <v>185</v>
       </c>
-      <c r="G30" t="s">
-        <v>15</v>
-      </c>
-      <c r="H30" t="s">
+      <c r="I30" t="s">
         <v>186</v>
       </c>
-      <c r="I30" t="s">
+      <c r="J30" t="s">
         <v>187</v>
-      </c>
-      <c r="J30" t="s">
-        <v>13</v>
       </c>
       <c r="K30" t="s">
         <v>188</v>
@@ -3485,7 +3500,7 @@
         <v>189</v>
       </c>
       <c r="B31" t="s">
-        <v>34</v>
+        <v>116</v>
       </c>
       <c r="C31" t="s">
         <v>13</v>
@@ -3509,106 +3524,106 @@
         <v>192</v>
       </c>
       <c r="J31" t="s">
+        <v>13</v>
+      </c>
+      <c r="K31" t="s">
         <v>193</v>
-      </c>
-      <c r="K31" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
+        <v>194</v>
+      </c>
+      <c r="B32" t="s">
+        <v>21</v>
+      </c>
+      <c r="C32" t="s">
+        <v>13</v>
+      </c>
+      <c r="D32" t="s">
+        <v>13</v>
+      </c>
+      <c r="E32" t="s">
+        <v>13</v>
+      </c>
+      <c r="F32" t="s">
         <v>195</v>
       </c>
-      <c r="B32" t="s">
+      <c r="G32" t="s">
+        <v>15</v>
+      </c>
+      <c r="H32" t="s">
         <v>196</v>
       </c>
-      <c r="C32" t="s">
-        <v>13</v>
-      </c>
-      <c r="D32" t="s">
-        <v>13</v>
-      </c>
-      <c r="E32" t="s">
-        <v>13</v>
-      </c>
-      <c r="F32" t="s">
+      <c r="I32" t="s">
         <v>197</v>
       </c>
-      <c r="G32" t="s">
-        <v>15</v>
-      </c>
-      <c r="H32" t="s">
+      <c r="J32" t="s">
         <v>198</v>
       </c>
-      <c r="I32" t="s">
+      <c r="K32" t="s">
         <v>199</v>
-      </c>
-      <c r="J32" t="s">
-        <v>200</v>
-      </c>
-      <c r="K32" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
+        <v>200</v>
+      </c>
+      <c r="B33" t="s">
+        <v>201</v>
+      </c>
+      <c r="C33" t="s">
+        <v>13</v>
+      </c>
+      <c r="D33" t="s">
+        <v>13</v>
+      </c>
+      <c r="E33" t="s">
+        <v>13</v>
+      </c>
+      <c r="F33" t="s">
         <v>202</v>
       </c>
-      <c r="B33" t="s">
+      <c r="G33" t="s">
+        <v>15</v>
+      </c>
+      <c r="H33" t="s">
         <v>203</v>
       </c>
-      <c r="C33" t="s">
-        <v>13</v>
-      </c>
-      <c r="D33" t="s">
-        <v>13</v>
-      </c>
-      <c r="E33" t="s">
-        <v>13</v>
-      </c>
-      <c r="F33" t="s">
+      <c r="I33" t="s">
         <v>204</v>
       </c>
-      <c r="G33" t="s">
-        <v>15</v>
-      </c>
-      <c r="H33" t="s">
+      <c r="J33" t="s">
         <v>205</v>
       </c>
-      <c r="I33" t="s">
+      <c r="K33" t="s">
         <v>206</v>
-      </c>
-      <c r="J33" t="s">
-        <v>207</v>
-      </c>
-      <c r="K33" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
+        <v>207</v>
+      </c>
+      <c r="B34" t="s">
+        <v>208</v>
+      </c>
+      <c r="C34" t="s">
+        <v>13</v>
+      </c>
+      <c r="D34" t="s">
+        <v>13</v>
+      </c>
+      <c r="E34" t="s">
+        <v>13</v>
+      </c>
+      <c r="F34" t="s">
         <v>209</v>
       </c>
-      <c r="B34" t="s">
-        <v>196</v>
-      </c>
-      <c r="C34" t="s">
-        <v>13</v>
-      </c>
-      <c r="D34" t="s">
-        <v>13</v>
-      </c>
-      <c r="E34" t="s">
-        <v>13</v>
-      </c>
-      <c r="F34" t="s">
+      <c r="G34" t="s">
+        <v>15</v>
+      </c>
+      <c r="H34" t="s">
         <v>210</v>
-      </c>
-      <c r="G34" t="s">
-        <v>15</v>
-      </c>
-      <c r="H34" t="s">
-        <v>198</v>
       </c>
       <c r="I34" t="s">
         <v>211</v>
@@ -3625,235 +3640,235 @@
         <v>214</v>
       </c>
       <c r="B35" t="s">
+        <v>201</v>
+      </c>
+      <c r="C35" t="s">
+        <v>13</v>
+      </c>
+      <c r="D35" t="s">
+        <v>13</v>
+      </c>
+      <c r="E35" t="s">
+        <v>13</v>
+      </c>
+      <c r="F35" t="s">
         <v>215</v>
       </c>
-      <c r="C35" t="s">
-        <v>13</v>
-      </c>
-      <c r="D35" t="s">
-        <v>13</v>
-      </c>
-      <c r="E35" t="s">
-        <v>13</v>
-      </c>
-      <c r="F35" t="s">
+      <c r="G35" t="s">
+        <v>15</v>
+      </c>
+      <c r="H35" t="s">
+        <v>203</v>
+      </c>
+      <c r="I35" t="s">
         <v>216</v>
       </c>
-      <c r="G35" t="s">
-        <v>15</v>
-      </c>
-      <c r="H35" t="s">
+      <c r="J35" t="s">
         <v>217</v>
       </c>
-      <c r="I35" t="s">
+      <c r="K35" t="s">
         <v>218</v>
-      </c>
-      <c r="J35" t="s">
-        <v>219</v>
-      </c>
-      <c r="K35" t="s">
-        <v>220</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
+        <v>219</v>
+      </c>
+      <c r="B36" t="s">
+        <v>220</v>
+      </c>
+      <c r="C36" t="s">
+        <v>13</v>
+      </c>
+      <c r="D36" t="s">
+        <v>13</v>
+      </c>
+      <c r="E36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F36" t="s">
         <v>221</v>
       </c>
-      <c r="B36" t="s">
+      <c r="G36" t="s">
+        <v>15</v>
+      </c>
+      <c r="H36" t="s">
         <v>222</v>
       </c>
-      <c r="C36" t="s">
-        <v>13</v>
-      </c>
-      <c r="D36" t="s">
-        <v>13</v>
-      </c>
-      <c r="E36" t="s">
-        <v>13</v>
-      </c>
-      <c r="F36" t="s">
+      <c r="I36" t="s">
         <v>223</v>
       </c>
-      <c r="G36" t="s">
-        <v>15</v>
-      </c>
-      <c r="H36" t="s">
-        <v>82</v>
-      </c>
-      <c r="I36" t="s">
+      <c r="J36" t="s">
         <v>224</v>
       </c>
-      <c r="J36" t="s">
+      <c r="K36" t="s">
         <v>225</v>
-      </c>
-      <c r="K36" t="s">
-        <v>226</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
+        <v>226</v>
+      </c>
+      <c r="B37" t="s">
         <v>227</v>
       </c>
-      <c r="B37" t="s">
+      <c r="C37" t="s">
+        <v>13</v>
+      </c>
+      <c r="D37" t="s">
+        <v>13</v>
+      </c>
+      <c r="E37" t="s">
+        <v>13</v>
+      </c>
+      <c r="F37" t="s">
         <v>228</v>
       </c>
-      <c r="C37" t="s">
-        <v>13</v>
-      </c>
-      <c r="D37" t="s">
-        <v>13</v>
-      </c>
-      <c r="E37" t="s">
-        <v>13</v>
-      </c>
-      <c r="F37" t="s">
+      <c r="G37" t="s">
+        <v>15</v>
+      </c>
+      <c r="H37" t="s">
+        <v>87</v>
+      </c>
+      <c r="I37" t="s">
         <v>229</v>
       </c>
-      <c r="G37" t="s">
-        <v>15</v>
-      </c>
-      <c r="H37" t="s">
+      <c r="J37" t="s">
         <v>230</v>
       </c>
-      <c r="I37" t="s">
+      <c r="K37" t="s">
         <v>231</v>
-      </c>
-      <c r="J37" t="s">
-        <v>232</v>
-      </c>
-      <c r="K37" t="s">
-        <v>233</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
+        <v>232</v>
+      </c>
+      <c r="B38" t="s">
+        <v>233</v>
+      </c>
+      <c r="C38" t="s">
+        <v>13</v>
+      </c>
+      <c r="D38" t="s">
+        <v>13</v>
+      </c>
+      <c r="E38" t="s">
+        <v>13</v>
+      </c>
+      <c r="F38" t="s">
         <v>234</v>
       </c>
-      <c r="B38" t="s">
+      <c r="G38" t="s">
+        <v>15</v>
+      </c>
+      <c r="H38" t="s">
         <v>235</v>
       </c>
-      <c r="C38" t="s">
+      <c r="I38" t="s">
         <v>236</v>
       </c>
-      <c r="D38" t="s">
-        <v>13</v>
-      </c>
-      <c r="E38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F38" t="s">
+      <c r="J38" t="s">
         <v>237</v>
       </c>
-      <c r="G38" t="s">
-        <v>15</v>
-      </c>
-      <c r="H38" t="s">
+      <c r="K38" t="s">
         <v>238</v>
-      </c>
-      <c r="I38" t="s">
-        <v>239</v>
-      </c>
-      <c r="J38" t="s">
-        <v>240</v>
-      </c>
-      <c r="K38" t="s">
-        <v>241</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
+        <v>239</v>
+      </c>
+      <c r="B39" t="s">
+        <v>240</v>
+      </c>
+      <c r="C39" t="s">
+        <v>241</v>
+      </c>
+      <c r="D39" t="s">
+        <v>13</v>
+      </c>
+      <c r="E39" t="s">
+        <v>13</v>
+      </c>
+      <c r="F39" t="s">
         <v>242</v>
       </c>
-      <c r="B39" t="s">
+      <c r="G39" t="s">
+        <v>15</v>
+      </c>
+      <c r="H39" t="s">
         <v>243</v>
       </c>
-      <c r="C39" t="s">
-        <v>13</v>
-      </c>
-      <c r="D39" t="s">
-        <v>13</v>
-      </c>
-      <c r="E39" t="s">
-        <v>13</v>
-      </c>
-      <c r="F39" t="s">
+      <c r="I39" t="s">
         <v>244</v>
       </c>
-      <c r="G39" t="s">
-        <v>15</v>
-      </c>
-      <c r="H39" t="s">
+      <c r="J39" t="s">
         <v>245</v>
       </c>
-      <c r="I39" t="s">
+      <c r="K39" t="s">
         <v>246</v>
-      </c>
-      <c r="J39" t="s">
-        <v>247</v>
-      </c>
-      <c r="K39" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
+        <v>247</v>
+      </c>
+      <c r="B40" t="s">
+        <v>248</v>
+      </c>
+      <c r="C40" t="s">
+        <v>13</v>
+      </c>
+      <c r="D40" t="s">
+        <v>13</v>
+      </c>
+      <c r="E40" t="s">
+        <v>13</v>
+      </c>
+      <c r="F40" t="s">
         <v>249</v>
       </c>
-      <c r="B40" t="s">
+      <c r="G40" t="s">
+        <v>15</v>
+      </c>
+      <c r="H40" t="s">
         <v>250</v>
       </c>
-      <c r="C40" t="s">
-        <v>13</v>
-      </c>
-      <c r="D40" t="s">
-        <v>13</v>
-      </c>
-      <c r="E40" t="s">
-        <v>13</v>
-      </c>
-      <c r="F40" t="s">
+      <c r="I40" t="s">
         <v>251</v>
       </c>
-      <c r="G40" t="s">
-        <v>15</v>
-      </c>
-      <c r="H40" t="s">
+      <c r="J40" t="s">
         <v>252</v>
       </c>
-      <c r="I40" t="s">
+      <c r="K40" t="s">
         <v>253</v>
-      </c>
-      <c r="J40" t="s">
-        <v>254</v>
-      </c>
-      <c r="K40" t="s">
-        <v>255</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
+        <v>254</v>
+      </c>
+      <c r="B41" t="s">
+        <v>255</v>
+      </c>
+      <c r="C41" t="s">
+        <v>13</v>
+      </c>
+      <c r="D41" t="s">
+        <v>13</v>
+      </c>
+      <c r="E41" t="s">
+        <v>13</v>
+      </c>
+      <c r="F41" t="s">
         <v>256</v>
       </c>
-      <c r="B41" t="s">
-        <v>104</v>
-      </c>
-      <c r="C41" t="s">
-        <v>13</v>
-      </c>
-      <c r="D41" t="s">
-        <v>13</v>
-      </c>
-      <c r="E41" t="s">
-        <v>13</v>
-      </c>
-      <c r="F41" t="s">
+      <c r="G41" t="s">
+        <v>15</v>
+      </c>
+      <c r="H41" t="s">
         <v>257</v>
-      </c>
-      <c r="G41" t="s">
-        <v>15</v>
-      </c>
-      <c r="H41" t="s">
-        <v>106</v>
       </c>
       <c r="I41" t="s">
         <v>258</v>
@@ -3870,7 +3885,7 @@
         <v>261</v>
       </c>
       <c r="B42" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="C42" t="s">
         <v>13</v>
@@ -3888,7 +3903,7 @@
         <v>15</v>
       </c>
       <c r="H42" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="I42" t="s">
         <v>263</v>
@@ -3905,7 +3920,7 @@
         <v>266</v>
       </c>
       <c r="B43" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="C43" t="s">
         <v>13</v>
@@ -3923,7 +3938,7 @@
         <v>15</v>
       </c>
       <c r="H43" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="I43" t="s">
         <v>268</v>
@@ -3940,42 +3955,42 @@
         <v>271</v>
       </c>
       <c r="B44" t="s">
+        <v>109</v>
+      </c>
+      <c r="C44" t="s">
+        <v>13</v>
+      </c>
+      <c r="D44" t="s">
+        <v>13</v>
+      </c>
+      <c r="E44" t="s">
+        <v>13</v>
+      </c>
+      <c r="F44" t="s">
         <v>272</v>
       </c>
-      <c r="C44" t="s">
-        <v>13</v>
-      </c>
-      <c r="D44" t="s">
-        <v>13</v>
-      </c>
-      <c r="E44" t="s">
-        <v>13</v>
-      </c>
-      <c r="F44" t="s">
+      <c r="G44" t="s">
+        <v>15</v>
+      </c>
+      <c r="H44" t="s">
+        <v>111</v>
+      </c>
+      <c r="I44" t="s">
         <v>273</v>
       </c>
-      <c r="G44" t="s">
-        <v>15</v>
-      </c>
-      <c r="H44" t="s">
+      <c r="J44" t="s">
         <v>274</v>
       </c>
-      <c r="I44" t="s">
+      <c r="K44" t="s">
         <v>275</v>
-      </c>
-      <c r="J44" t="s">
-        <v>13</v>
-      </c>
-      <c r="K44" t="s">
-        <v>276</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
+        <v>276</v>
+      </c>
+      <c r="B45" t="s">
         <v>277</v>
-      </c>
-      <c r="B45" t="s">
-        <v>104</v>
       </c>
       <c r="C45" t="s">
         <v>13</v>
@@ -3993,13 +4008,13 @@
         <v>15</v>
       </c>
       <c r="H45" t="s">
-        <v>106</v>
+        <v>279</v>
       </c>
       <c r="I45" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="J45" t="s">
-        <v>280</v>
+        <v>13</v>
       </c>
       <c r="K45" t="s">
         <v>281</v>
@@ -4010,7 +4025,7 @@
         <v>282</v>
       </c>
       <c r="B46" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="C46" t="s">
         <v>13</v>
@@ -4028,7 +4043,7 @@
         <v>15</v>
       </c>
       <c r="H46" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="I46" t="s">
         <v>284</v>
@@ -4045,235 +4060,235 @@
         <v>287</v>
       </c>
       <c r="B47" t="s">
+        <v>109</v>
+      </c>
+      <c r="C47" t="s">
+        <v>13</v>
+      </c>
+      <c r="D47" t="s">
+        <v>13</v>
+      </c>
+      <c r="E47" t="s">
+        <v>13</v>
+      </c>
+      <c r="F47" t="s">
         <v>288</v>
       </c>
-      <c r="C47" t="s">
-        <v>13</v>
-      </c>
-      <c r="D47" t="s">
-        <v>13</v>
-      </c>
-      <c r="E47" t="s">
-        <v>13</v>
-      </c>
-      <c r="F47" t="s">
+      <c r="G47" t="s">
+        <v>15</v>
+      </c>
+      <c r="H47" t="s">
+        <v>111</v>
+      </c>
+      <c r="I47" t="s">
         <v>289</v>
       </c>
-      <c r="G47" t="s">
-        <v>15</v>
-      </c>
-      <c r="H47" t="s">
+      <c r="J47" t="s">
         <v>290</v>
       </c>
-      <c r="I47" t="s">
+      <c r="K47" t="s">
         <v>291</v>
-      </c>
-      <c r="J47" t="s">
-        <v>292</v>
-      </c>
-      <c r="K47" t="s">
-        <v>293</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
+        <v>292</v>
+      </c>
+      <c r="B48" t="s">
+        <v>293</v>
+      </c>
+      <c r="C48" t="s">
+        <v>13</v>
+      </c>
+      <c r="D48" t="s">
+        <v>13</v>
+      </c>
+      <c r="E48" t="s">
+        <v>13</v>
+      </c>
+      <c r="F48" t="s">
         <v>294</v>
       </c>
-      <c r="B48" t="s">
+      <c r="G48" t="s">
+        <v>15</v>
+      </c>
+      <c r="H48" t="s">
         <v>295</v>
       </c>
-      <c r="C48" t="s">
-        <v>13</v>
-      </c>
-      <c r="D48" t="s">
-        <v>13</v>
-      </c>
-      <c r="E48" t="s">
-        <v>13</v>
-      </c>
-      <c r="F48" t="s">
+      <c r="I48" t="s">
         <v>296</v>
       </c>
-      <c r="G48" t="s">
-        <v>15</v>
-      </c>
-      <c r="H48" t="s">
+      <c r="J48" t="s">
         <v>297</v>
       </c>
-      <c r="I48" t="s">
+      <c r="K48" t="s">
         <v>298</v>
-      </c>
-      <c r="J48" t="s">
-        <v>299</v>
-      </c>
-      <c r="K48" t="s">
-        <v>300</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
+        <v>299</v>
+      </c>
+      <c r="B49" t="s">
+        <v>300</v>
+      </c>
+      <c r="C49" t="s">
+        <v>13</v>
+      </c>
+      <c r="D49" t="s">
+        <v>13</v>
+      </c>
+      <c r="E49" t="s">
+        <v>13</v>
+      </c>
+      <c r="F49" t="s">
         <v>301</v>
       </c>
-      <c r="B49" t="s">
+      <c r="G49" t="s">
+        <v>15</v>
+      </c>
+      <c r="H49" t="s">
         <v>302</v>
       </c>
-      <c r="C49" t="s">
-        <v>13</v>
-      </c>
-      <c r="D49" t="s">
-        <v>13</v>
-      </c>
-      <c r="E49" t="s">
-        <v>13</v>
-      </c>
-      <c r="F49" t="s">
+      <c r="I49" t="s">
         <v>303</v>
       </c>
-      <c r="G49" t="s">
-        <v>15</v>
-      </c>
-      <c r="H49" t="s">
+      <c r="J49" t="s">
         <v>304</v>
       </c>
-      <c r="I49" t="s">
+      <c r="K49" t="s">
         <v>305</v>
-      </c>
-      <c r="J49" t="s">
-        <v>306</v>
-      </c>
-      <c r="K49" t="s">
-        <v>307</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
+        <v>306</v>
+      </c>
+      <c r="B50" t="s">
+        <v>307</v>
+      </c>
+      <c r="C50" t="s">
+        <v>13</v>
+      </c>
+      <c r="D50" t="s">
+        <v>13</v>
+      </c>
+      <c r="E50" t="s">
+        <v>13</v>
+      </c>
+      <c r="F50" t="s">
         <v>308</v>
       </c>
-      <c r="B50" t="s">
+      <c r="G50" t="s">
+        <v>15</v>
+      </c>
+      <c r="H50" t="s">
         <v>309</v>
       </c>
-      <c r="C50" t="s">
-        <v>13</v>
-      </c>
-      <c r="D50" t="s">
-        <v>13</v>
-      </c>
-      <c r="E50" t="s">
-        <v>13</v>
-      </c>
-      <c r="F50" t="s">
+      <c r="I50" t="s">
         <v>310</v>
       </c>
-      <c r="G50" t="s">
-        <v>15</v>
-      </c>
-      <c r="H50" t="s">
-        <v>297</v>
-      </c>
-      <c r="I50" t="s">
+      <c r="J50" t="s">
         <v>311</v>
       </c>
-      <c r="J50" t="s">
+      <c r="K50" t="s">
         <v>312</v>
-      </c>
-      <c r="K50" t="s">
-        <v>313</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
+        <v>313</v>
+      </c>
+      <c r="B51" t="s">
         <v>314</v>
       </c>
-      <c r="B51" t="s">
+      <c r="C51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51" t="s">
+        <v>13</v>
+      </c>
+      <c r="E51" t="s">
+        <v>13</v>
+      </c>
+      <c r="F51" t="s">
         <v>315</v>
       </c>
-      <c r="C51" t="s">
-        <v>13</v>
-      </c>
-      <c r="D51" t="s">
-        <v>13</v>
-      </c>
-      <c r="E51" t="s">
-        <v>13</v>
-      </c>
-      <c r="F51" t="s">
+      <c r="G51" t="s">
+        <v>15</v>
+      </c>
+      <c r="H51" t="s">
+        <v>302</v>
+      </c>
+      <c r="I51" t="s">
         <v>316</v>
       </c>
-      <c r="G51" t="s">
-        <v>15</v>
-      </c>
-      <c r="H51" t="s">
+      <c r="J51" t="s">
         <v>317</v>
       </c>
-      <c r="I51" t="s">
+      <c r="K51" t="s">
         <v>318</v>
-      </c>
-      <c r="J51" t="s">
-        <v>319</v>
-      </c>
-      <c r="K51" t="s">
-        <v>320</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
+        <v>319</v>
+      </c>
+      <c r="B52" t="s">
+        <v>320</v>
+      </c>
+      <c r="C52" t="s">
+        <v>13</v>
+      </c>
+      <c r="D52" t="s">
+        <v>13</v>
+      </c>
+      <c r="E52" t="s">
+        <v>13</v>
+      </c>
+      <c r="F52" t="s">
         <v>321</v>
       </c>
-      <c r="B52" t="s">
-        <v>104</v>
-      </c>
-      <c r="C52" t="s">
-        <v>13</v>
-      </c>
-      <c r="D52" t="s">
-        <v>13</v>
-      </c>
-      <c r="E52" t="s">
-        <v>13</v>
-      </c>
-      <c r="F52" t="s">
+      <c r="G52" t="s">
+        <v>15</v>
+      </c>
+      <c r="H52" t="s">
         <v>322</v>
       </c>
-      <c r="G52" t="s">
-        <v>15</v>
-      </c>
-      <c r="H52" t="s">
+      <c r="I52" t="s">
         <v>323</v>
       </c>
-      <c r="I52" t="s">
+      <c r="J52" t="s">
         <v>324</v>
       </c>
-      <c r="J52" t="s">
+      <c r="K52" t="s">
         <v>325</v>
-      </c>
-      <c r="K52" t="s">
-        <v>326</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
+        <v>326</v>
+      </c>
+      <c r="B53" t="s">
+        <v>109</v>
+      </c>
+      <c r="C53" t="s">
+        <v>13</v>
+      </c>
+      <c r="D53" t="s">
+        <v>13</v>
+      </c>
+      <c r="E53" t="s">
+        <v>13</v>
+      </c>
+      <c r="F53" t="s">
         <v>327</v>
       </c>
-      <c r="B53" t="s">
-        <v>104</v>
-      </c>
-      <c r="C53" t="s">
-        <v>13</v>
-      </c>
-      <c r="D53" t="s">
-        <v>13</v>
-      </c>
-      <c r="E53" t="s">
-        <v>13</v>
-      </c>
-      <c r="F53" t="s">
+      <c r="G53" t="s">
+        <v>15</v>
+      </c>
+      <c r="H53" t="s">
         <v>328</v>
-      </c>
-      <c r="G53" t="s">
-        <v>15</v>
-      </c>
-      <c r="H53" t="s">
-        <v>323</v>
       </c>
       <c r="I53" t="s">
         <v>329</v>
@@ -4290,112 +4305,112 @@
         <v>332</v>
       </c>
       <c r="B54" t="s">
+        <v>109</v>
+      </c>
+      <c r="C54" t="s">
+        <v>13</v>
+      </c>
+      <c r="D54" t="s">
+        <v>13</v>
+      </c>
+      <c r="E54" t="s">
+        <v>13</v>
+      </c>
+      <c r="F54" t="s">
         <v>333</v>
       </c>
-      <c r="C54" t="s">
-        <v>13</v>
-      </c>
-      <c r="D54" t="s">
-        <v>13</v>
-      </c>
-      <c r="E54" t="s">
-        <v>13</v>
-      </c>
-      <c r="F54" t="s">
+      <c r="G54" t="s">
+        <v>15</v>
+      </c>
+      <c r="H54" t="s">
+        <v>328</v>
+      </c>
+      <c r="I54" t="s">
         <v>334</v>
       </c>
-      <c r="G54" t="s">
-        <v>15</v>
-      </c>
-      <c r="H54" t="s">
-        <v>323</v>
-      </c>
-      <c r="I54" t="s">
+      <c r="J54" t="s">
         <v>335</v>
       </c>
-      <c r="J54" t="s">
+      <c r="K54" t="s">
         <v>336</v>
-      </c>
-      <c r="K54" t="s">
-        <v>337</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
+        <v>337</v>
+      </c>
+      <c r="B55" t="s">
         <v>338</v>
       </c>
-      <c r="B55" t="s">
+      <c r="C55" t="s">
+        <v>13</v>
+      </c>
+      <c r="D55" t="s">
+        <v>13</v>
+      </c>
+      <c r="E55" t="s">
+        <v>13</v>
+      </c>
+      <c r="F55" t="s">
         <v>339</v>
       </c>
-      <c r="C55" t="s">
-        <v>13</v>
-      </c>
-      <c r="D55" t="s">
-        <v>13</v>
-      </c>
-      <c r="E55" t="s">
-        <v>13</v>
-      </c>
-      <c r="F55" t="s">
+      <c r="G55" t="s">
+        <v>15</v>
+      </c>
+      <c r="H55" t="s">
+        <v>328</v>
+      </c>
+      <c r="I55" t="s">
         <v>340</v>
       </c>
-      <c r="G55" t="s">
-        <v>15</v>
-      </c>
-      <c r="H55" t="s">
-        <v>217</v>
-      </c>
-      <c r="I55" t="s">
+      <c r="J55" t="s">
         <v>341</v>
       </c>
-      <c r="J55" t="s">
+      <c r="K55" t="s">
         <v>342</v>
-      </c>
-      <c r="K55" t="s">
-        <v>343</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
+        <v>343</v>
+      </c>
+      <c r="B56" t="s">
         <v>344</v>
       </c>
-      <c r="B56" t="s">
+      <c r="C56" t="s">
+        <v>13</v>
+      </c>
+      <c r="D56" t="s">
+        <v>13</v>
+      </c>
+      <c r="E56" t="s">
+        <v>13</v>
+      </c>
+      <c r="F56" t="s">
         <v>345</v>
       </c>
-      <c r="C56" t="s">
-        <v>13</v>
-      </c>
-      <c r="D56" t="s">
-        <v>13</v>
-      </c>
-      <c r="E56" t="s">
-        <v>13</v>
-      </c>
-      <c r="F56" t="s">
+      <c r="G56" t="s">
+        <v>15</v>
+      </c>
+      <c r="H56" t="s">
+        <v>222</v>
+      </c>
+      <c r="I56" t="s">
         <v>346</v>
       </c>
-      <c r="G56" t="s">
-        <v>15</v>
-      </c>
-      <c r="H56" t="s">
-        <v>230</v>
-      </c>
-      <c r="I56" t="s">
+      <c r="J56" t="s">
         <v>347</v>
       </c>
-      <c r="J56" t="s">
+      <c r="K56" t="s">
         <v>348</v>
-      </c>
-      <c r="K56" t="s">
-        <v>349</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
+        <v>349</v>
+      </c>
+      <c r="B57" t="s">
         <v>350</v>
-      </c>
-      <c r="B57" t="s">
-        <v>345</v>
       </c>
       <c r="C57" t="s">
         <v>13</v>
@@ -4413,7 +4428,7 @@
         <v>15</v>
       </c>
       <c r="H57" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="I57" t="s">
         <v>352</v>
@@ -4430,7 +4445,7 @@
         <v>355</v>
       </c>
       <c r="B58" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
       <c r="C58" t="s">
         <v>13</v>
@@ -4448,7 +4463,7 @@
         <v>15</v>
       </c>
       <c r="H58" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="I58" t="s">
         <v>357</v>
@@ -4465,77 +4480,77 @@
         <v>360</v>
       </c>
       <c r="B59" t="s">
+        <v>350</v>
+      </c>
+      <c r="C59" t="s">
+        <v>13</v>
+      </c>
+      <c r="D59" t="s">
+        <v>13</v>
+      </c>
+      <c r="E59" t="s">
+        <v>13</v>
+      </c>
+      <c r="F59" t="s">
         <v>361</v>
       </c>
-      <c r="C59" t="s">
-        <v>13</v>
-      </c>
-      <c r="D59" t="s">
-        <v>13</v>
-      </c>
-      <c r="E59" t="s">
-        <v>13</v>
-      </c>
-      <c r="F59" t="s">
+      <c r="G59" t="s">
+        <v>15</v>
+      </c>
+      <c r="H59" t="s">
+        <v>235</v>
+      </c>
+      <c r="I59" t="s">
         <v>362</v>
       </c>
-      <c r="G59" t="s">
-        <v>15</v>
-      </c>
-      <c r="H59" t="s">
-        <v>230</v>
-      </c>
-      <c r="I59" t="s">
+      <c r="J59" t="s">
         <v>363</v>
       </c>
-      <c r="J59" t="s">
+      <c r="K59" t="s">
         <v>364</v>
-      </c>
-      <c r="K59" t="s">
-        <v>365</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
+        <v>365</v>
+      </c>
+      <c r="B60" t="s">
         <v>366</v>
       </c>
-      <c r="B60" t="s">
+      <c r="C60" t="s">
+        <v>13</v>
+      </c>
+      <c r="D60" t="s">
+        <v>13</v>
+      </c>
+      <c r="E60" t="s">
+        <v>13</v>
+      </c>
+      <c r="F60" t="s">
         <v>367</v>
       </c>
-      <c r="C60" t="s">
-        <v>13</v>
-      </c>
-      <c r="D60" t="s">
-        <v>13</v>
-      </c>
-      <c r="E60" t="s">
-        <v>13</v>
-      </c>
-      <c r="F60" t="s">
+      <c r="G60" t="s">
+        <v>15</v>
+      </c>
+      <c r="H60" t="s">
+        <v>235</v>
+      </c>
+      <c r="I60" t="s">
         <v>368</v>
       </c>
-      <c r="G60" t="s">
-        <v>15</v>
-      </c>
-      <c r="H60" t="s">
-        <v>230</v>
-      </c>
-      <c r="I60" t="s">
+      <c r="J60" t="s">
         <v>369</v>
       </c>
-      <c r="J60" t="s">
+      <c r="K60" t="s">
         <v>370</v>
-      </c>
-      <c r="K60" t="s">
-        <v>371</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
+        <v>371</v>
+      </c>
+      <c r="B61" t="s">
         <v>372</v>
-      </c>
-      <c r="B61" t="s">
-        <v>345</v>
       </c>
       <c r="C61" t="s">
         <v>13</v>
@@ -4553,7 +4568,7 @@
         <v>15</v>
       </c>
       <c r="H61" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="I61" t="s">
         <v>374</v>
@@ -4570,7 +4585,7 @@
         <v>377</v>
       </c>
       <c r="B62" t="s">
-        <v>104</v>
+        <v>350</v>
       </c>
       <c r="C62" t="s">
         <v>13</v>
@@ -4588,94 +4603,94 @@
         <v>15</v>
       </c>
       <c r="H62" t="s">
+        <v>235</v>
+      </c>
+      <c r="I62" t="s">
         <v>379</v>
       </c>
-      <c r="I62" t="s">
+      <c r="J62" t="s">
         <v>380</v>
       </c>
-      <c r="J62" t="s">
+      <c r="K62" t="s">
         <v>381</v>
-      </c>
-      <c r="K62" t="s">
-        <v>382</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
+        <v>382</v>
+      </c>
+      <c r="B63" t="s">
+        <v>109</v>
+      </c>
+      <c r="C63" t="s">
+        <v>13</v>
+      </c>
+      <c r="D63" t="s">
+        <v>13</v>
+      </c>
+      <c r="E63" t="s">
+        <v>13</v>
+      </c>
+      <c r="F63" t="s">
         <v>383</v>
       </c>
-      <c r="B63" t="s">
+      <c r="G63" t="s">
+        <v>15</v>
+      </c>
+      <c r="H63" t="s">
         <v>384</v>
       </c>
-      <c r="C63" t="s">
-        <v>13</v>
-      </c>
-      <c r="D63" t="s">
-        <v>13</v>
-      </c>
-      <c r="E63" t="s">
-        <v>13</v>
-      </c>
-      <c r="F63" t="s">
+      <c r="I63" t="s">
         <v>385</v>
       </c>
-      <c r="G63" t="s">
-        <v>15</v>
-      </c>
-      <c r="H63" t="s">
-        <v>217</v>
-      </c>
-      <c r="I63" t="s">
+      <c r="J63" t="s">
         <v>386</v>
       </c>
-      <c r="J63" t="s">
+      <c r="K63" t="s">
         <v>387</v>
-      </c>
-      <c r="K63" t="s">
-        <v>388</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
+        <v>388</v>
+      </c>
+      <c r="B64" t="s">
         <v>389</v>
       </c>
-      <c r="B64" t="s">
+      <c r="C64" t="s">
+        <v>13</v>
+      </c>
+      <c r="D64" t="s">
+        <v>13</v>
+      </c>
+      <c r="E64" t="s">
+        <v>13</v>
+      </c>
+      <c r="F64" t="s">
         <v>390</v>
       </c>
-      <c r="C64" t="s">
-        <v>13</v>
-      </c>
-      <c r="D64" t="s">
-        <v>13</v>
-      </c>
-      <c r="E64" t="s">
-        <v>13</v>
-      </c>
-      <c r="F64" t="s">
+      <c r="G64" t="s">
+        <v>15</v>
+      </c>
+      <c r="H64" t="s">
+        <v>222</v>
+      </c>
+      <c r="I64" t="s">
         <v>391</v>
       </c>
-      <c r="G64" t="s">
-        <v>15</v>
-      </c>
-      <c r="H64" t="s">
-        <v>217</v>
-      </c>
-      <c r="I64" t="s">
+      <c r="J64" t="s">
         <v>392</v>
       </c>
-      <c r="J64" t="s">
+      <c r="K64" t="s">
         <v>393</v>
-      </c>
-      <c r="K64" t="s">
-        <v>394</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
+        <v>394</v>
+      </c>
+      <c r="B65" t="s">
         <v>395</v>
-      </c>
-      <c r="B65" t="s">
-        <v>384</v>
       </c>
       <c r="C65" t="s">
         <v>13</v>
@@ -4693,7 +4708,7 @@
         <v>15</v>
       </c>
       <c r="H65" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="I65" t="s">
         <v>397</v>
@@ -4710,7 +4725,7 @@
         <v>400</v>
       </c>
       <c r="B66" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="C66" t="s">
         <v>13</v>
@@ -4728,7 +4743,7 @@
         <v>15</v>
       </c>
       <c r="H66" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="I66" t="s">
         <v>402</v>
@@ -4745,182 +4760,182 @@
         <v>405</v>
       </c>
       <c r="B67" t="s">
-        <v>34</v>
+        <v>395</v>
       </c>
       <c r="C67" t="s">
+        <v>13</v>
+      </c>
+      <c r="D67" t="s">
+        <v>13</v>
+      </c>
+      <c r="E67" t="s">
+        <v>13</v>
+      </c>
+      <c r="F67" t="s">
         <v>406</v>
       </c>
-      <c r="D67" t="s">
-        <v>13</v>
-      </c>
-      <c r="E67" t="s">
-        <v>13</v>
-      </c>
-      <c r="F67" t="s">
+      <c r="G67" t="s">
+        <v>15</v>
+      </c>
+      <c r="H67" t="s">
+        <v>222</v>
+      </c>
+      <c r="I67" t="s">
         <v>407</v>
       </c>
-      <c r="G67" t="s">
-        <v>15</v>
-      </c>
-      <c r="H67" t="s">
+      <c r="J67" t="s">
         <v>408</v>
       </c>
-      <c r="I67" t="s">
+      <c r="K67" t="s">
         <v>409</v>
-      </c>
-      <c r="J67" t="s">
-        <v>410</v>
-      </c>
-      <c r="K67" t="s">
-        <v>411</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
+        <v>410</v>
+      </c>
+      <c r="B68" t="s">
+        <v>21</v>
+      </c>
+      <c r="C68" t="s">
+        <v>411</v>
+      </c>
+      <c r="D68" t="s">
+        <v>13</v>
+      </c>
+      <c r="E68" t="s">
+        <v>13</v>
+      </c>
+      <c r="F68" t="s">
         <v>412</v>
       </c>
-      <c r="B68" t="s">
-        <v>34</v>
-      </c>
-      <c r="C68" t="s">
+      <c r="G68" t="s">
+        <v>15</v>
+      </c>
+      <c r="H68" t="s">
         <v>413</v>
       </c>
-      <c r="D68" t="s">
-        <v>13</v>
-      </c>
-      <c r="E68" t="s">
-        <v>13</v>
-      </c>
-      <c r="F68" t="s">
+      <c r="I68" t="s">
         <v>414</v>
       </c>
-      <c r="G68" t="s">
-        <v>15</v>
-      </c>
-      <c r="H68" t="s">
-        <v>408</v>
-      </c>
-      <c r="I68" t="s">
+      <c r="J68" t="s">
         <v>415</v>
       </c>
-      <c r="J68" t="s">
+      <c r="K68" t="s">
         <v>416</v>
-      </c>
-      <c r="K68" t="s">
-        <v>417</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
+        <v>417</v>
+      </c>
+      <c r="B69" t="s">
+        <v>21</v>
+      </c>
+      <c r="C69" t="s">
         <v>418</v>
       </c>
-      <c r="B69" t="s">
-        <v>34</v>
-      </c>
-      <c r="C69" t="s">
+      <c r="D69" t="s">
+        <v>13</v>
+      </c>
+      <c r="E69" t="s">
+        <v>13</v>
+      </c>
+      <c r="F69" t="s">
         <v>419</v>
       </c>
-      <c r="D69" t="s">
-        <v>13</v>
-      </c>
-      <c r="E69" t="s">
+      <c r="G69" t="s">
+        <v>15</v>
+      </c>
+      <c r="H69" t="s">
+        <v>413</v>
+      </c>
+      <c r="I69" t="s">
         <v>420</v>
       </c>
-      <c r="F69" t="s">
+      <c r="J69" t="s">
         <v>421</v>
       </c>
-      <c r="G69" t="s">
-        <v>15</v>
-      </c>
-      <c r="H69" t="s">
+      <c r="K69" t="s">
         <v>422</v>
-      </c>
-      <c r="I69" t="s">
-        <v>423</v>
-      </c>
-      <c r="J69" t="s">
-        <v>424</v>
-      </c>
-      <c r="K69" t="s">
-        <v>425</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
+        <v>423</v>
+      </c>
+      <c r="B70" t="s">
+        <v>21</v>
+      </c>
+      <c r="C70" t="s">
+        <v>424</v>
+      </c>
+      <c r="D70" t="s">
+        <v>13</v>
+      </c>
+      <c r="E70" t="s">
+        <v>425</v>
+      </c>
+      <c r="F70" t="s">
         <v>426</v>
       </c>
-      <c r="B70" t="s">
+      <c r="G70" t="s">
+        <v>15</v>
+      </c>
+      <c r="H70" t="s">
         <v>427</v>
       </c>
-      <c r="C70" t="s">
-        <v>13</v>
-      </c>
-      <c r="D70" t="s">
-        <v>13</v>
-      </c>
-      <c r="E70" t="s">
-        <v>13</v>
-      </c>
-      <c r="F70" t="s">
+      <c r="I70" t="s">
         <v>428</v>
       </c>
-      <c r="G70" t="s">
-        <v>15</v>
-      </c>
-      <c r="H70" t="s">
+      <c r="J70" t="s">
         <v>429</v>
       </c>
-      <c r="I70" t="s">
+      <c r="K70" t="s">
         <v>430</v>
-      </c>
-      <c r="J70" t="s">
-        <v>431</v>
-      </c>
-      <c r="K70" t="s">
-        <v>432</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
+        <v>431</v>
+      </c>
+      <c r="B71" t="s">
+        <v>432</v>
+      </c>
+      <c r="C71" t="s">
+        <v>13</v>
+      </c>
+      <c r="D71" t="s">
+        <v>13</v>
+      </c>
+      <c r="E71" t="s">
+        <v>13</v>
+      </c>
+      <c r="F71" t="s">
         <v>433</v>
       </c>
-      <c r="B71" t="s">
+      <c r="G71" t="s">
+        <v>15</v>
+      </c>
+      <c r="H71" t="s">
         <v>434</v>
       </c>
-      <c r="C71" t="s">
-        <v>13</v>
-      </c>
-      <c r="D71" t="s">
-        <v>13</v>
-      </c>
-      <c r="E71" t="s">
-        <v>13</v>
-      </c>
-      <c r="F71" t="s">
+      <c r="I71" t="s">
         <v>435</v>
       </c>
-      <c r="G71" t="s">
-        <v>15</v>
-      </c>
-      <c r="H71" t="s">
-        <v>429</v>
-      </c>
-      <c r="I71" t="s">
+      <c r="J71" t="s">
         <v>436</v>
       </c>
-      <c r="J71" t="s">
+      <c r="K71" t="s">
         <v>437</v>
-      </c>
-      <c r="K71" t="s">
-        <v>438</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
+        <v>438</v>
+      </c>
+      <c r="B72" t="s">
         <v>439</v>
-      </c>
-      <c r="B72" t="s">
-        <v>434</v>
       </c>
       <c r="C72" t="s">
         <v>13</v>
@@ -4938,7 +4953,7 @@
         <v>15</v>
       </c>
       <c r="H72" t="s">
-        <v>429</v>
+        <v>434</v>
       </c>
       <c r="I72" t="s">
         <v>441</v>
@@ -4955,7 +4970,7 @@
         <v>444</v>
       </c>
       <c r="B73" t="s">
-        <v>434</v>
+        <v>439</v>
       </c>
       <c r="C73" t="s">
         <v>13</v>
@@ -4973,7 +4988,7 @@
         <v>15</v>
       </c>
       <c r="H73" t="s">
-        <v>429</v>
+        <v>434</v>
       </c>
       <c r="I73" t="s">
         <v>446</v>
@@ -4990,95 +5005,95 @@
         <v>449</v>
       </c>
       <c r="B74" t="s">
+        <v>439</v>
+      </c>
+      <c r="C74" t="s">
+        <v>13</v>
+      </c>
+      <c r="D74" t="s">
+        <v>13</v>
+      </c>
+      <c r="E74" t="s">
+        <v>13</v>
+      </c>
+      <c r="F74" t="s">
         <v>450</v>
       </c>
-      <c r="C74" t="s">
-        <v>13</v>
-      </c>
-      <c r="D74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E74" t="s">
-        <v>13</v>
-      </c>
-      <c r="F74" t="s">
+      <c r="G74" t="s">
+        <v>15</v>
+      </c>
+      <c r="H74" t="s">
+        <v>434</v>
+      </c>
+      <c r="I74" t="s">
         <v>451</v>
       </c>
-      <c r="G74" t="s">
-        <v>15</v>
-      </c>
-      <c r="H74" t="s">
-        <v>429</v>
-      </c>
-      <c r="I74" t="s">
+      <c r="J74" t="s">
         <v>452</v>
       </c>
-      <c r="J74" t="s">
+      <c r="K74" t="s">
         <v>453</v>
-      </c>
-      <c r="K74" t="s">
-        <v>454</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
+        <v>454</v>
+      </c>
+      <c r="B75" t="s">
         <v>455</v>
       </c>
-      <c r="B75" t="s">
+      <c r="C75" t="s">
+        <v>13</v>
+      </c>
+      <c r="D75" t="s">
+        <v>13</v>
+      </c>
+      <c r="E75" t="s">
+        <v>13</v>
+      </c>
+      <c r="F75" t="s">
         <v>456</v>
       </c>
-      <c r="C75" t="s">
-        <v>13</v>
-      </c>
-      <c r="D75" t="s">
-        <v>13</v>
-      </c>
-      <c r="E75" t="s">
-        <v>13</v>
-      </c>
-      <c r="F75" t="s">
+      <c r="G75" t="s">
+        <v>15</v>
+      </c>
+      <c r="H75" t="s">
+        <v>434</v>
+      </c>
+      <c r="I75" t="s">
         <v>457</v>
       </c>
-      <c r="G75" t="s">
-        <v>15</v>
-      </c>
-      <c r="H75" t="s">
+      <c r="J75" t="s">
         <v>458</v>
       </c>
-      <c r="I75" t="s">
+      <c r="K75" t="s">
         <v>459</v>
-      </c>
-      <c r="J75" t="s">
-        <v>460</v>
-      </c>
-      <c r="K75" t="s">
-        <v>461</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
+        <v>460</v>
+      </c>
+      <c r="B76" t="s">
+        <v>461</v>
+      </c>
+      <c r="C76" t="s">
+        <v>13</v>
+      </c>
+      <c r="D76" t="s">
+        <v>13</v>
+      </c>
+      <c r="E76" t="s">
+        <v>13</v>
+      </c>
+      <c r="F76" t="s">
         <v>462</v>
       </c>
-      <c r="B76" t="s">
-        <v>456</v>
-      </c>
-      <c r="C76" t="s">
-        <v>13</v>
-      </c>
-      <c r="D76" t="s">
-        <v>13</v>
-      </c>
-      <c r="E76" t="s">
-        <v>13</v>
-      </c>
-      <c r="F76" t="s">
+      <c r="G76" t="s">
+        <v>15</v>
+      </c>
+      <c r="H76" t="s">
         <v>463</v>
-      </c>
-      <c r="G76" t="s">
-        <v>15</v>
-      </c>
-      <c r="H76" t="s">
-        <v>458</v>
       </c>
       <c r="I76" t="s">
         <v>464</v>
@@ -5095,7 +5110,7 @@
         <v>467</v>
       </c>
       <c r="B77" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
       <c r="C77" t="s">
         <v>13</v>
@@ -5113,7 +5128,7 @@
         <v>15</v>
       </c>
       <c r="H77" t="s">
-        <v>458</v>
+        <v>463</v>
       </c>
       <c r="I77" t="s">
         <v>469</v>
@@ -5130,7 +5145,7 @@
         <v>472</v>
       </c>
       <c r="B78" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
       <c r="C78" t="s">
         <v>13</v>
@@ -5148,7 +5163,7 @@
         <v>15</v>
       </c>
       <c r="H78" t="s">
-        <v>458</v>
+        <v>463</v>
       </c>
       <c r="I78" t="s">
         <v>474</v>
@@ -5157,15 +5172,15 @@
         <v>475</v>
       </c>
       <c r="K78" t="s">
-        <v>170</v>
+        <v>476</v>
       </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="B79" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
       <c r="C79" t="s">
         <v>13</v>
@@ -5177,30 +5192,30 @@
         <v>13</v>
       </c>
       <c r="F79" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="G79" t="s">
         <v>15</v>
       </c>
       <c r="H79" t="s">
-        <v>458</v>
+        <v>463</v>
       </c>
       <c r="I79" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="J79" t="s">
-        <v>13</v>
+        <v>480</v>
       </c>
       <c r="K79" t="s">
-        <v>479</v>
+        <v>175</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="B80" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
       <c r="C80" t="s">
         <v>13</v>
@@ -5212,30 +5227,30 @@
         <v>13</v>
       </c>
       <c r="F80" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="G80" t="s">
         <v>15</v>
       </c>
       <c r="H80" t="s">
-        <v>458</v>
+        <v>463</v>
       </c>
       <c r="I80" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="J80" t="s">
         <v>13</v>
       </c>
       <c r="K80" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="B81" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
       <c r="C81" t="s">
         <v>13</v>
@@ -5247,30 +5262,30 @@
         <v>13</v>
       </c>
       <c r="F81" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="G81" t="s">
         <v>15</v>
       </c>
       <c r="H81" t="s">
-        <v>458</v>
+        <v>463</v>
       </c>
       <c r="I81" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="J81" t="s">
         <v>13</v>
       </c>
       <c r="K81" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="B82" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
       <c r="C82" t="s">
         <v>13</v>
@@ -5282,19 +5297,19 @@
         <v>13</v>
       </c>
       <c r="F82" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="G82" t="s">
         <v>15</v>
       </c>
       <c r="H82" t="s">
-        <v>458</v>
+        <v>463</v>
       </c>
       <c r="I82" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="J82" t="s">
-        <v>491</v>
+        <v>13</v>
       </c>
       <c r="K82" t="s">
         <v>492</v>
@@ -5305,7 +5320,7 @@
         <v>493</v>
       </c>
       <c r="B83" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
       <c r="C83" t="s">
         <v>13</v>
@@ -5323,7 +5338,7 @@
         <v>15</v>
       </c>
       <c r="H83" t="s">
-        <v>458</v>
+        <v>463</v>
       </c>
       <c r="I83" t="s">
         <v>495</v>
@@ -5340,7 +5355,7 @@
         <v>498</v>
       </c>
       <c r="B84" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
       <c r="C84" t="s">
         <v>13</v>
@@ -5358,24 +5373,24 @@
         <v>15</v>
       </c>
       <c r="H84" t="s">
-        <v>458</v>
+        <v>463</v>
       </c>
       <c r="I84" t="s">
         <v>500</v>
       </c>
       <c r="J84" t="s">
-        <v>13</v>
+        <v>501</v>
       </c>
       <c r="K84" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="B85" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
       <c r="C85" t="s">
         <v>13</v>
@@ -5387,19 +5402,19 @@
         <v>13</v>
       </c>
       <c r="F85" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="G85" t="s">
         <v>15</v>
       </c>
       <c r="H85" t="s">
-        <v>458</v>
+        <v>463</v>
       </c>
       <c r="I85" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="J85" t="s">
-        <v>505</v>
+        <v>13</v>
       </c>
       <c r="K85" t="s">
         <v>506</v>
@@ -5410,7 +5425,7 @@
         <v>507</v>
       </c>
       <c r="B86" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
       <c r="C86" t="s">
         <v>13</v>
@@ -5428,7 +5443,7 @@
         <v>15</v>
       </c>
       <c r="H86" t="s">
-        <v>458</v>
+        <v>463</v>
       </c>
       <c r="I86" t="s">
         <v>509</v>
@@ -5445,7 +5460,7 @@
         <v>512</v>
       </c>
       <c r="B87" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
       <c r="C87" t="s">
         <v>13</v>
@@ -5463,24 +5478,24 @@
         <v>15</v>
       </c>
       <c r="H87" t="s">
-        <v>458</v>
+        <v>463</v>
       </c>
       <c r="I87" t="s">
         <v>514</v>
       </c>
       <c r="J87" t="s">
-        <v>13</v>
+        <v>515</v>
       </c>
       <c r="K87" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
     </row>
     <row r="88" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="B88" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
       <c r="C88" t="s">
         <v>13</v>
@@ -5492,19 +5507,19 @@
         <v>13</v>
       </c>
       <c r="F88" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="G88" t="s">
         <v>15</v>
       </c>
       <c r="H88" t="s">
-        <v>458</v>
+        <v>463</v>
       </c>
       <c r="I88" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="J88" t="s">
-        <v>519</v>
+        <v>13</v>
       </c>
       <c r="K88" t="s">
         <v>520</v>
@@ -5515,7 +5530,7 @@
         <v>521</v>
       </c>
       <c r="B89" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
       <c r="C89" t="s">
         <v>13</v>
@@ -5533,7 +5548,7 @@
         <v>15</v>
       </c>
       <c r="H89" t="s">
-        <v>458</v>
+        <v>463</v>
       </c>
       <c r="I89" t="s">
         <v>523</v>
@@ -5550,7 +5565,7 @@
         <v>526</v>
       </c>
       <c r="B90" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
       <c r="C90" t="s">
         <v>13</v>
@@ -5568,24 +5583,24 @@
         <v>15</v>
       </c>
       <c r="H90" t="s">
-        <v>458</v>
+        <v>463</v>
       </c>
       <c r="I90" t="s">
         <v>528</v>
       </c>
       <c r="J90" t="s">
-        <v>13</v>
+        <v>529</v>
       </c>
       <c r="K90" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
     </row>
     <row r="91" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="B91" t="s">
-        <v>104</v>
+        <v>461</v>
       </c>
       <c r="C91" t="s">
         <v>13</v>
@@ -5597,118 +5612,118 @@
         <v>13</v>
       </c>
       <c r="F91" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="G91" t="s">
         <v>15</v>
       </c>
       <c r="H91" t="s">
-        <v>532</v>
+        <v>463</v>
       </c>
       <c r="I91" t="s">
         <v>533</v>
       </c>
       <c r="J91" t="s">
+        <v>13</v>
+      </c>
+      <c r="K91" t="s">
         <v>534</v>
-      </c>
-      <c r="K91" t="s">
-        <v>535</v>
       </c>
     </row>
     <row r="92" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
+        <v>535</v>
+      </c>
+      <c r="B92" t="s">
+        <v>109</v>
+      </c>
+      <c r="C92" t="s">
+        <v>13</v>
+      </c>
+      <c r="D92" t="s">
+        <v>13</v>
+      </c>
+      <c r="E92" t="s">
+        <v>13</v>
+      </c>
+      <c r="F92" t="s">
         <v>536</v>
       </c>
-      <c r="B92" t="s">
+      <c r="G92" t="s">
+        <v>15</v>
+      </c>
+      <c r="H92" t="s">
         <v>537</v>
       </c>
-      <c r="C92" t="s">
-        <v>13</v>
-      </c>
-      <c r="D92" t="s">
-        <v>13</v>
-      </c>
-      <c r="E92" t="s">
-        <v>13</v>
-      </c>
-      <c r="F92" t="s">
+      <c r="I92" t="s">
         <v>538</v>
       </c>
-      <c r="G92" t="s">
-        <v>15</v>
-      </c>
-      <c r="H92" t="s">
-        <v>323</v>
-      </c>
-      <c r="I92" t="s">
+      <c r="J92" t="s">
         <v>539</v>
       </c>
-      <c r="J92" t="s">
+      <c r="K92" t="s">
         <v>540</v>
-      </c>
-      <c r="K92" t="s">
-        <v>541</v>
       </c>
     </row>
     <row r="93" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
+        <v>541</v>
+      </c>
+      <c r="B93" t="s">
         <v>542</v>
       </c>
-      <c r="B93" t="s">
+      <c r="C93" t="s">
+        <v>13</v>
+      </c>
+      <c r="D93" t="s">
+        <v>13</v>
+      </c>
+      <c r="E93" t="s">
+        <v>13</v>
+      </c>
+      <c r="F93" t="s">
         <v>543</v>
       </c>
-      <c r="C93" t="s">
-        <v>13</v>
-      </c>
-      <c r="D93" t="s">
-        <v>13</v>
-      </c>
-      <c r="E93" t="s">
-        <v>13</v>
-      </c>
-      <c r="F93" t="s">
+      <c r="G93" t="s">
+        <v>15</v>
+      </c>
+      <c r="H93" t="s">
+        <v>328</v>
+      </c>
+      <c r="I93" t="s">
         <v>544</v>
       </c>
-      <c r="G93" t="s">
-        <v>15</v>
-      </c>
-      <c r="H93" t="s">
+      <c r="J93" t="s">
         <v>545</v>
       </c>
-      <c r="I93" t="s">
+      <c r="K93" t="s">
         <v>546</v>
-      </c>
-      <c r="J93" t="s">
-        <v>547</v>
-      </c>
-      <c r="K93" t="s">
-        <v>548</v>
       </c>
     </row>
     <row r="94" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
+        <v>547</v>
+      </c>
+      <c r="B94" t="s">
+        <v>548</v>
+      </c>
+      <c r="C94" t="s">
+        <v>13</v>
+      </c>
+      <c r="D94" t="s">
+        <v>13</v>
+      </c>
+      <c r="E94" t="s">
+        <v>13</v>
+      </c>
+      <c r="F94" t="s">
         <v>549</v>
       </c>
-      <c r="B94" t="s">
-        <v>333</v>
-      </c>
-      <c r="C94" t="s">
-        <v>13</v>
-      </c>
-      <c r="D94" t="s">
-        <v>13</v>
-      </c>
-      <c r="E94" t="s">
-        <v>13</v>
-      </c>
-      <c r="F94" t="s">
+      <c r="G94" t="s">
+        <v>15</v>
+      </c>
+      <c r="H94" t="s">
         <v>550</v>
-      </c>
-      <c r="G94" t="s">
-        <v>15</v>
-      </c>
-      <c r="H94" t="s">
-        <v>323</v>
       </c>
       <c r="I94" t="s">
         <v>551</v>
@@ -5725,42 +5740,42 @@
         <v>554</v>
       </c>
       <c r="B95" t="s">
+        <v>338</v>
+      </c>
+      <c r="C95" t="s">
+        <v>13</v>
+      </c>
+      <c r="D95" t="s">
+        <v>13</v>
+      </c>
+      <c r="E95" t="s">
+        <v>13</v>
+      </c>
+      <c r="F95" t="s">
         <v>555</v>
       </c>
-      <c r="C95" t="s">
-        <v>13</v>
-      </c>
-      <c r="D95" t="s">
-        <v>13</v>
-      </c>
-      <c r="E95" t="s">
-        <v>13</v>
-      </c>
-      <c r="F95" t="s">
+      <c r="G95" t="s">
+        <v>15</v>
+      </c>
+      <c r="H95" t="s">
+        <v>328</v>
+      </c>
+      <c r="I95" t="s">
         <v>556</v>
       </c>
-      <c r="G95" t="s">
-        <v>15</v>
-      </c>
-      <c r="H95" t="s">
-        <v>323</v>
-      </c>
-      <c r="I95" t="s">
+      <c r="J95" t="s">
         <v>557</v>
       </c>
-      <c r="J95" t="s">
+      <c r="K95" t="s">
         <v>558</v>
-      </c>
-      <c r="K95" t="s">
-        <v>559</v>
       </c>
     </row>
     <row r="96" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
+        <v>559</v>
+      </c>
+      <c r="B96" t="s">
         <v>560</v>
-      </c>
-      <c r="B96" t="s">
-        <v>537</v>
       </c>
       <c r="C96" t="s">
         <v>13</v>
@@ -5778,7 +5793,7 @@
         <v>15</v>
       </c>
       <c r="H96" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="I96" t="s">
         <v>562</v>
@@ -5795,7 +5810,7 @@
         <v>565</v>
       </c>
       <c r="B97" t="s">
-        <v>104</v>
+        <v>542</v>
       </c>
       <c r="C97" t="s">
         <v>13</v>
@@ -5813,7 +5828,7 @@
         <v>15</v>
       </c>
       <c r="H97" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="I97" t="s">
         <v>567</v>
@@ -5830,7 +5845,7 @@
         <v>570</v>
       </c>
       <c r="B98" t="s">
-        <v>543</v>
+        <v>109</v>
       </c>
       <c r="C98" t="s">
         <v>13</v>
@@ -5848,7 +5863,7 @@
         <v>15</v>
       </c>
       <c r="H98" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="I98" t="s">
         <v>572</v>
@@ -5865,42 +5880,42 @@
         <v>575</v>
       </c>
       <c r="B99" t="s">
+        <v>548</v>
+      </c>
+      <c r="C99" t="s">
+        <v>13</v>
+      </c>
+      <c r="D99" t="s">
+        <v>13</v>
+      </c>
+      <c r="E99" t="s">
+        <v>13</v>
+      </c>
+      <c r="F99" t="s">
         <v>576</v>
       </c>
-      <c r="C99" t="s">
-        <v>13</v>
-      </c>
-      <c r="D99" t="s">
-        <v>13</v>
-      </c>
-      <c r="E99" t="s">
-        <v>13</v>
-      </c>
-      <c r="F99" t="s">
+      <c r="G99" t="s">
+        <v>15</v>
+      </c>
+      <c r="H99" t="s">
+        <v>328</v>
+      </c>
+      <c r="I99" t="s">
         <v>577</v>
       </c>
-      <c r="G99" t="s">
-        <v>15</v>
-      </c>
-      <c r="H99" t="s">
-        <v>545</v>
-      </c>
-      <c r="I99" t="s">
+      <c r="J99" t="s">
         <v>578</v>
       </c>
-      <c r="J99" t="s">
+      <c r="K99" t="s">
         <v>579</v>
-      </c>
-      <c r="K99" t="s">
-        <v>580</v>
       </c>
     </row>
     <row r="100" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
+        <v>580</v>
+      </c>
+      <c r="B100" t="s">
         <v>581</v>
-      </c>
-      <c r="B100" t="s">
-        <v>543</v>
       </c>
       <c r="C100" t="s">
         <v>13</v>
@@ -5918,7 +5933,7 @@
         <v>15</v>
       </c>
       <c r="H100" t="s">
-        <v>323</v>
+        <v>550</v>
       </c>
       <c r="I100" t="s">
         <v>583</v>
@@ -5935,7 +5950,7 @@
         <v>586</v>
       </c>
       <c r="B101" t="s">
-        <v>537</v>
+        <v>548</v>
       </c>
       <c r="C101" t="s">
         <v>13</v>
@@ -5953,7 +5968,7 @@
         <v>15</v>
       </c>
       <c r="H101" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="I101" t="s">
         <v>588</v>
@@ -5970,42 +5985,42 @@
         <v>591</v>
       </c>
       <c r="B102" t="s">
+        <v>542</v>
+      </c>
+      <c r="C102" t="s">
+        <v>13</v>
+      </c>
+      <c r="D102" t="s">
+        <v>13</v>
+      </c>
+      <c r="E102" t="s">
+        <v>13</v>
+      </c>
+      <c r="F102" t="s">
         <v>592</v>
       </c>
-      <c r="C102" t="s">
-        <v>13</v>
-      </c>
-      <c r="D102" t="s">
-        <v>13</v>
-      </c>
-      <c r="E102" t="s">
-        <v>13</v>
-      </c>
-      <c r="F102" t="s">
+      <c r="G102" t="s">
+        <v>15</v>
+      </c>
+      <c r="H102" t="s">
+        <v>328</v>
+      </c>
+      <c r="I102" t="s">
         <v>593</v>
       </c>
-      <c r="G102" t="s">
-        <v>15</v>
-      </c>
-      <c r="H102" t="s">
-        <v>323</v>
-      </c>
-      <c r="I102" t="s">
+      <c r="J102" t="s">
         <v>594</v>
       </c>
-      <c r="J102" t="s">
+      <c r="K102" t="s">
         <v>595</v>
-      </c>
-      <c r="K102" t="s">
-        <v>596</v>
       </c>
     </row>
     <row r="103" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
+        <v>596</v>
+      </c>
+      <c r="B103" t="s">
         <v>597</v>
-      </c>
-      <c r="B103" t="s">
-        <v>543</v>
       </c>
       <c r="C103" t="s">
         <v>13</v>
@@ -6023,7 +6038,7 @@
         <v>15</v>
       </c>
       <c r="H103" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="I103" t="s">
         <v>599</v>
@@ -6040,7 +6055,7 @@
         <v>602</v>
       </c>
       <c r="B104" t="s">
-        <v>537</v>
+        <v>548</v>
       </c>
       <c r="C104" t="s">
         <v>13</v>
@@ -6058,42 +6073,42 @@
         <v>15</v>
       </c>
       <c r="H104" t="s">
+        <v>328</v>
+      </c>
+      <c r="I104" t="s">
         <v>604</v>
       </c>
-      <c r="I104" t="s">
+      <c r="J104" t="s">
         <v>605</v>
       </c>
-      <c r="J104" t="s">
+      <c r="K104" t="s">
         <v>606</v>
-      </c>
-      <c r="K104" t="s">
-        <v>607</v>
       </c>
     </row>
     <row r="105" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
+        <v>607</v>
+      </c>
+      <c r="B105" t="s">
+        <v>542</v>
+      </c>
+      <c r="C105" t="s">
+        <v>13</v>
+      </c>
+      <c r="D105" t="s">
+        <v>13</v>
+      </c>
+      <c r="E105" t="s">
+        <v>13</v>
+      </c>
+      <c r="F105" t="s">
         <v>608</v>
       </c>
-      <c r="B105" t="s">
-        <v>543</v>
-      </c>
-      <c r="C105" t="s">
-        <v>13</v>
-      </c>
-      <c r="D105" t="s">
-        <v>13</v>
-      </c>
-      <c r="E105" t="s">
-        <v>13</v>
-      </c>
-      <c r="F105" t="s">
+      <c r="G105" t="s">
+        <v>15</v>
+      </c>
+      <c r="H105" t="s">
         <v>609</v>
-      </c>
-      <c r="G105" t="s">
-        <v>15</v>
-      </c>
-      <c r="H105" t="s">
-        <v>545</v>
       </c>
       <c r="I105" t="s">
         <v>610</v>
@@ -6110,7 +6125,7 @@
         <v>613</v>
       </c>
       <c r="B106" t="s">
-        <v>543</v>
+        <v>548</v>
       </c>
       <c r="C106" t="s">
         <v>13</v>
@@ -6128,7 +6143,7 @@
         <v>15</v>
       </c>
       <c r="H106" t="s">
-        <v>323</v>
+        <v>550</v>
       </c>
       <c r="I106" t="s">
         <v>615</v>
@@ -6145,7 +6160,7 @@
         <v>618</v>
       </c>
       <c r="B107" t="s">
-        <v>537</v>
+        <v>548</v>
       </c>
       <c r="C107" t="s">
         <v>13</v>
@@ -6163,7 +6178,7 @@
         <v>15</v>
       </c>
       <c r="H107" t="s">
-        <v>604</v>
+        <v>328</v>
       </c>
       <c r="I107" t="s">
         <v>620</v>
@@ -6180,7 +6195,7 @@
         <v>623</v>
       </c>
       <c r="B108" t="s">
-        <v>104</v>
+        <v>542</v>
       </c>
       <c r="C108" t="s">
         <v>13</v>
@@ -6198,7 +6213,7 @@
         <v>15</v>
       </c>
       <c r="H108" t="s">
-        <v>379</v>
+        <v>609</v>
       </c>
       <c r="I108" t="s">
         <v>625</v>
@@ -6215,7 +6230,7 @@
         <v>628</v>
       </c>
       <c r="B109" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="C109" t="s">
         <v>13</v>
@@ -6233,7 +6248,7 @@
         <v>15</v>
       </c>
       <c r="H109" t="s">
-        <v>379</v>
+        <v>384</v>
       </c>
       <c r="I109" t="s">
         <v>630</v>
@@ -6250,7 +6265,7 @@
         <v>633</v>
       </c>
       <c r="B110" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="C110" t="s">
         <v>13</v>
@@ -6268,7 +6283,7 @@
         <v>15</v>
       </c>
       <c r="H110" t="s">
-        <v>379</v>
+        <v>384</v>
       </c>
       <c r="I110" t="s">
         <v>635</v>
@@ -6285,7 +6300,7 @@
         <v>638</v>
       </c>
       <c r="B111" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="C111" t="s">
         <v>13</v>
@@ -6303,7 +6318,7 @@
         <v>15</v>
       </c>
       <c r="H111" t="s">
-        <v>379</v>
+        <v>384</v>
       </c>
       <c r="I111" t="s">
         <v>640</v>
@@ -6320,7 +6335,7 @@
         <v>643</v>
       </c>
       <c r="B112" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="C112" t="s">
         <v>13</v>
@@ -6338,7 +6353,7 @@
         <v>15</v>
       </c>
       <c r="H112" t="s">
-        <v>532</v>
+        <v>384</v>
       </c>
       <c r="I112" t="s">
         <v>645</v>
@@ -6355,7 +6370,7 @@
         <v>648</v>
       </c>
       <c r="B113" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="C113" t="s">
         <v>13</v>
@@ -6373,7 +6388,7 @@
         <v>15</v>
       </c>
       <c r="H113" t="s">
-        <v>379</v>
+        <v>537</v>
       </c>
       <c r="I113" t="s">
         <v>650</v>
@@ -6390,51 +6405,51 @@
         <v>653</v>
       </c>
       <c r="B114" t="s">
+        <v>109</v>
+      </c>
+      <c r="C114" t="s">
+        <v>13</v>
+      </c>
+      <c r="D114" t="s">
+        <v>13</v>
+      </c>
+      <c r="E114" t="s">
+        <v>13</v>
+      </c>
+      <c r="F114" t="s">
         <v>654</v>
       </c>
-      <c r="C114" t="s">
-        <v>406</v>
-      </c>
-      <c r="D114" t="s">
-        <v>13</v>
-      </c>
-      <c r="E114" t="s">
+      <c r="G114" t="s">
+        <v>15</v>
+      </c>
+      <c r="H114" t="s">
+        <v>384</v>
+      </c>
+      <c r="I114" t="s">
         <v>655</v>
       </c>
-      <c r="F114" t="s">
+      <c r="J114" t="s">
         <v>656</v>
       </c>
-      <c r="G114" t="s">
-        <v>15</v>
-      </c>
-      <c r="H114" t="s">
-        <v>422</v>
-      </c>
-      <c r="I114" t="s">
+      <c r="K114" t="s">
         <v>657</v>
-      </c>
-      <c r="J114" t="s">
-        <v>658</v>
-      </c>
-      <c r="K114" t="s">
-        <v>659</v>
       </c>
     </row>
     <row r="115" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
+        <v>658</v>
+      </c>
+      <c r="B115" t="s">
+        <v>659</v>
+      </c>
+      <c r="C115" t="s">
+        <v>411</v>
+      </c>
+      <c r="D115" t="s">
+        <v>13</v>
+      </c>
+      <c r="E115" t="s">
         <v>660</v>
-      </c>
-      <c r="B115" t="s">
-        <v>654</v>
-      </c>
-      <c r="C115" t="s">
-        <v>413</v>
-      </c>
-      <c r="D115" t="s">
-        <v>13</v>
-      </c>
-      <c r="E115" t="s">
-        <v>655</v>
       </c>
       <c r="F115" t="s">
         <v>661</v>
@@ -6443,7 +6458,7 @@
         <v>15</v>
       </c>
       <c r="H115" t="s">
-        <v>422</v>
+        <v>427</v>
       </c>
       <c r="I115" t="s">
         <v>662</v>
@@ -6460,34 +6475,69 @@
         <v>665</v>
       </c>
       <c r="B116" t="s">
+        <v>659</v>
+      </c>
+      <c r="C116" t="s">
+        <v>418</v>
+      </c>
+      <c r="D116" t="s">
+        <v>13</v>
+      </c>
+      <c r="E116" t="s">
+        <v>660</v>
+      </c>
+      <c r="F116" t="s">
         <v>666</v>
       </c>
-      <c r="C116" t="s">
+      <c r="G116" t="s">
+        <v>15</v>
+      </c>
+      <c r="H116" t="s">
+        <v>427</v>
+      </c>
+      <c r="I116" t="s">
         <v>667</v>
       </c>
-      <c r="D116" t="s">
-        <v>13</v>
-      </c>
-      <c r="E116" t="s">
+      <c r="J116" t="s">
         <v>668</v>
       </c>
-      <c r="F116" t="s">
+      <c r="K116" t="s">
         <v>669</v>
       </c>
-      <c r="G116" t="s">
-        <v>15</v>
-      </c>
-      <c r="H116" t="s">
-        <v>422</v>
-      </c>
-      <c r="I116" t="s">
+    </row>
+    <row r="117" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
         <v>670</v>
       </c>
-      <c r="J116" t="s">
+      <c r="B117" t="s">
         <v>671</v>
       </c>
-      <c r="K116" t="s">
+      <c r="C117" t="s">
         <v>672</v>
+      </c>
+      <c r="D117" t="s">
+        <v>13</v>
+      </c>
+      <c r="E117" t="s">
+        <v>673</v>
+      </c>
+      <c r="F117" t="s">
+        <v>674</v>
+      </c>
+      <c r="G117" t="s">
+        <v>15</v>
+      </c>
+      <c r="H117" t="s">
+        <v>427</v>
+      </c>
+      <c r="I117" t="s">
+        <v>675</v>
+      </c>
+      <c r="J117" t="s">
+        <v>676</v>
+      </c>
+      <c r="K117" t="s">
+        <v>677</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
/contact: "form below" links to the form (#110)
The source links "form below" to #contact, which no element there has. The
importer now keeps the link as #contact-form, and form-minimal-light gives
each form its sheet's name as its id (contact-form, fraud-form,
news-alert-form) unless the page already uses it.

Co-authored-by: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-contact.report.xlsx
+++ b/tools/importer/reports/import-contact.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1275" uniqueCount="673">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1286" uniqueCount="678">
   <si>
     <t>_reportFile</t>
   </si>
@@ -73,6 +73,27 @@
     <t>https://www.highmark.com/because-life</t>
   </si>
   <si>
+    <t>contact-thank-you.report.json</t>
+  </si>
+  <si>
+    <t>[]</t>
+  </si>
+  <si>
+    <t>contact-thank-you</t>
+  </si>
+  <si>
+    <t>fraud-thank-you</t>
+  </si>
+  <si>
+    <t>2026-10-14T08:30:39.378Z</t>
+  </si>
+  <si>
+    <t>Thank You</t>
+  </si>
+  <si>
+    <t>https://www.highmark.com/contact-thank-you</t>
+  </si>
+  <si>
     <t>contact.report.json</t>
   </si>
   <si>
@@ -82,7 +103,7 @@
     <t>contact</t>
   </si>
   <si>
-    <t>2026-10-14T08:30:32.469Z</t>
+    <t>2026-10-14T09:06:59.963Z</t>
   </si>
   <si>
     <t>Contact Highmark</t>
@@ -113,12 +134,6 @@
   </si>
   <si>
     <t>fraud-thank-you.report.json</t>
-  </si>
-  <si>
-    <t>[]</t>
-  </si>
-  <si>
-    <t>fraud-thank-you</t>
   </si>
   <si>
     <t>2026-10-14T07:13:24.168Z</t>
@@ -2418,7 +2433,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K116"/>
+  <dimension ref="A1:K117"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="50" customWidth="1"/>
@@ -2523,24 +2538,24 @@
         <v>15</v>
       </c>
       <c r="H3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C4" t="s">
         <v>13</v>
@@ -2552,7 +2567,7 @@
         <v>13</v>
       </c>
       <c r="F4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G4" t="s">
         <v>15</v>
@@ -2593,24 +2608,24 @@
         <v>15</v>
       </c>
       <c r="H5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="I5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="J5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="K5" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B6" t="s">
-        <v>40</v>
+        <v>21</v>
       </c>
       <c r="C6" t="s">
         <v>13</v>
@@ -2622,112 +2637,112 @@
         <v>13</v>
       </c>
       <c r="F6" t="s">
+        <v>23</v>
+      </c>
+      <c r="G6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I6" t="s">
         <v>41</v>
       </c>
-      <c r="G6" t="s">
-        <v>15</v>
-      </c>
-      <c r="H6" t="s">
+      <c r="J6" t="s">
         <v>42</v>
       </c>
-      <c r="I6" t="s">
+      <c r="K6" t="s">
         <v>43</v>
-      </c>
-      <c r="J6" t="s">
-        <v>44</v>
-      </c>
-      <c r="K6" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>44</v>
+      </c>
+      <c r="B7" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" t="s">
         <v>46</v>
       </c>
-      <c r="B7" t="s">
+      <c r="G7" t="s">
+        <v>15</v>
+      </c>
+      <c r="H7" t="s">
         <v>47</v>
       </c>
-      <c r="C7" t="s">
-        <v>13</v>
-      </c>
-      <c r="D7" t="s">
-        <v>13</v>
-      </c>
-      <c r="E7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F7" t="s">
+      <c r="I7" t="s">
         <v>48</v>
       </c>
-      <c r="G7" t="s">
-        <v>15</v>
-      </c>
-      <c r="H7" t="s">
-        <v>16</v>
-      </c>
-      <c r="I7" t="s">
+      <c r="J7" t="s">
         <v>49</v>
       </c>
-      <c r="J7" t="s">
+      <c r="K7" t="s">
         <v>50</v>
-      </c>
-      <c r="K7" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B8" t="s">
         <v>52</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" t="s">
         <v>53</v>
       </c>
-      <c r="C8" t="s">
-        <v>13</v>
-      </c>
-      <c r="D8" t="s">
-        <v>13</v>
-      </c>
-      <c r="E8" t="s">
-        <v>13</v>
-      </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
+        <v>15</v>
+      </c>
+      <c r="H8" t="s">
+        <v>16</v>
+      </c>
+      <c r="I8" t="s">
         <v>54</v>
       </c>
-      <c r="G8" t="s">
-        <v>15</v>
-      </c>
-      <c r="H8" t="s">
+      <c r="J8" t="s">
         <v>55</v>
       </c>
-      <c r="I8" t="s">
+      <c r="K8" t="s">
         <v>56</v>
-      </c>
-      <c r="J8" t="s">
-        <v>57</v>
-      </c>
-      <c r="K8" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>57</v>
+      </c>
+      <c r="B9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F9" t="s">
         <v>59</v>
-      </c>
-      <c r="B9" t="s">
-        <v>34</v>
-      </c>
-      <c r="C9" t="s">
-        <v>13</v>
-      </c>
-      <c r="D9" t="s">
-        <v>13</v>
-      </c>
-      <c r="E9" t="s">
-        <v>13</v>
-      </c>
-      <c r="F9" t="s">
-        <v>60</v>
       </c>
       <c r="G9" t="s">
         <v>15</v>
@@ -2750,7 +2765,7 @@
         <v>64</v>
       </c>
       <c r="B10" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="C10" t="s">
         <v>13</v>
@@ -2774,18 +2789,18 @@
         <v>66</v>
       </c>
       <c r="J10" t="s">
-        <v>13</v>
+        <v>67</v>
       </c>
       <c r="K10" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B11" t="s">
-        <v>69</v>
+        <v>21</v>
       </c>
       <c r="C11" t="s">
         <v>13</v>
@@ -2803,42 +2818,42 @@
         <v>15</v>
       </c>
       <c r="H11" t="s">
+        <v>70</v>
+      </c>
+      <c r="I11" t="s">
         <v>71</v>
       </c>
-      <c r="I11" t="s">
+      <c r="J11" t="s">
+        <v>13</v>
+      </c>
+      <c r="K11" t="s">
         <v>72</v>
-      </c>
-      <c r="J11" t="s">
-        <v>73</v>
-      </c>
-      <c r="K11" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>73</v>
+      </c>
+      <c r="B12" t="s">
+        <v>74</v>
+      </c>
+      <c r="C12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D12" t="s">
+        <v>13</v>
+      </c>
+      <c r="E12" t="s">
+        <v>13</v>
+      </c>
+      <c r="F12" t="s">
         <v>75</v>
       </c>
-      <c r="B12" t="s">
-        <v>34</v>
-      </c>
-      <c r="C12" t="s">
-        <v>13</v>
-      </c>
-      <c r="D12" t="s">
-        <v>13</v>
-      </c>
-      <c r="E12" t="s">
-        <v>13</v>
-      </c>
-      <c r="F12" t="s">
+      <c r="G12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H12" t="s">
         <v>76</v>
-      </c>
-      <c r="G12" t="s">
-        <v>15</v>
-      </c>
-      <c r="H12" t="s">
-        <v>71</v>
       </c>
       <c r="I12" t="s">
         <v>77</v>
@@ -2855,7 +2870,7 @@
         <v>80</v>
       </c>
       <c r="B13" t="s">
-        <v>47</v>
+        <v>21</v>
       </c>
       <c r="C13" t="s">
         <v>13</v>
@@ -2873,118 +2888,118 @@
         <v>15</v>
       </c>
       <c r="H13" t="s">
+        <v>76</v>
+      </c>
+      <c r="I13" t="s">
         <v>82</v>
       </c>
-      <c r="I13" t="s">
+      <c r="J13" t="s">
         <v>83</v>
       </c>
-      <c r="J13" t="s">
+      <c r="K13" t="s">
         <v>84</v>
-      </c>
-      <c r="K13" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>85</v>
+      </c>
+      <c r="B14" t="s">
+        <v>52</v>
+      </c>
+      <c r="C14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D14" t="s">
+        <v>13</v>
+      </c>
+      <c r="E14" t="s">
+        <v>13</v>
+      </c>
+      <c r="F14" t="s">
         <v>86</v>
       </c>
-      <c r="B14" t="s">
+      <c r="G14" t="s">
+        <v>15</v>
+      </c>
+      <c r="H14" t="s">
         <v>87</v>
       </c>
-      <c r="C14" t="s">
-        <v>13</v>
-      </c>
-      <c r="D14" t="s">
-        <v>13</v>
-      </c>
-      <c r="E14" t="s">
-        <v>13</v>
-      </c>
-      <c r="F14" t="s">
+      <c r="I14" t="s">
         <v>88</v>
       </c>
-      <c r="G14" t="s">
-        <v>15</v>
-      </c>
-      <c r="H14" t="s">
-        <v>16</v>
-      </c>
-      <c r="I14" t="s">
+      <c r="J14" t="s">
         <v>89</v>
       </c>
-      <c r="J14" t="s">
+      <c r="K14" t="s">
         <v>90</v>
-      </c>
-      <c r="K14" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>91</v>
+      </c>
+      <c r="B15" t="s">
         <v>92</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
+        <v>13</v>
+      </c>
+      <c r="D15" t="s">
+        <v>13</v>
+      </c>
+      <c r="E15" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15" t="s">
         <v>93</v>
       </c>
-      <c r="C15" t="s">
-        <v>13</v>
-      </c>
-      <c r="D15" t="s">
-        <v>13</v>
-      </c>
-      <c r="E15" t="s">
-        <v>13</v>
-      </c>
-      <c r="F15" t="s">
+      <c r="G15" t="s">
+        <v>15</v>
+      </c>
+      <c r="H15" t="s">
+        <v>16</v>
+      </c>
+      <c r="I15" t="s">
         <v>94</v>
       </c>
-      <c r="G15" t="s">
-        <v>15</v>
-      </c>
-      <c r="H15" t="s">
-        <v>42</v>
-      </c>
-      <c r="I15" t="s">
+      <c r="J15" t="s">
         <v>95</v>
       </c>
-      <c r="J15" t="s">
+      <c r="K15" t="s">
         <v>96</v>
-      </c>
-      <c r="K15" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>97</v>
+      </c>
+      <c r="B16" t="s">
         <v>98</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
+        <v>13</v>
+      </c>
+      <c r="D16" t="s">
+        <v>13</v>
+      </c>
+      <c r="E16" t="s">
+        <v>13</v>
+      </c>
+      <c r="F16" t="s">
         <v>99</v>
       </c>
-      <c r="C16" t="s">
-        <v>13</v>
-      </c>
-      <c r="D16" t="s">
-        <v>13</v>
-      </c>
-      <c r="E16" t="s">
-        <v>13</v>
-      </c>
-      <c r="F16" t="s">
+      <c r="G16" t="s">
+        <v>15</v>
+      </c>
+      <c r="H16" t="s">
+        <v>47</v>
+      </c>
+      <c r="I16" t="s">
         <v>100</v>
       </c>
-      <c r="G16" t="s">
-        <v>15</v>
-      </c>
-      <c r="H16" t="s">
-        <v>100</v>
-      </c>
-      <c r="I16" t="s">
+      <c r="J16" t="s">
         <v>101</v>
-      </c>
-      <c r="J16" t="s">
-        <v>13</v>
       </c>
       <c r="K16" t="s">
         <v>102</v>
@@ -3013,77 +3028,77 @@
         <v>15</v>
       </c>
       <c r="H17" t="s">
+        <v>105</v>
+      </c>
+      <c r="I17" t="s">
         <v>106</v>
       </c>
-      <c r="I17" t="s">
+      <c r="J17" t="s">
+        <v>13</v>
+      </c>
+      <c r="K17" t="s">
         <v>107</v>
-      </c>
-      <c r="J17" t="s">
-        <v>108</v>
-      </c>
-      <c r="K17" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>108</v>
+      </c>
+      <c r="B18" t="s">
+        <v>109</v>
+      </c>
+      <c r="C18" t="s">
+        <v>13</v>
+      </c>
+      <c r="D18" t="s">
+        <v>13</v>
+      </c>
+      <c r="E18" t="s">
+        <v>13</v>
+      </c>
+      <c r="F18" t="s">
         <v>110</v>
       </c>
-      <c r="B18" t="s">
+      <c r="G18" t="s">
+        <v>15</v>
+      </c>
+      <c r="H18" t="s">
         <v>111</v>
       </c>
-      <c r="C18" t="s">
-        <v>13</v>
-      </c>
-      <c r="D18" t="s">
-        <v>13</v>
-      </c>
-      <c r="E18" t="s">
-        <v>13</v>
-      </c>
-      <c r="F18" t="s">
+      <c r="I18" t="s">
         <v>112</v>
       </c>
-      <c r="G18" t="s">
-        <v>15</v>
-      </c>
-      <c r="H18" t="s">
+      <c r="J18" t="s">
         <v>113</v>
       </c>
-      <c r="I18" t="s">
+      <c r="K18" t="s">
         <v>114</v>
-      </c>
-      <c r="J18" t="s">
-        <v>115</v>
-      </c>
-      <c r="K18" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>115</v>
+      </c>
+      <c r="B19" t="s">
+        <v>116</v>
+      </c>
+      <c r="C19" t="s">
+        <v>13</v>
+      </c>
+      <c r="D19" t="s">
+        <v>13</v>
+      </c>
+      <c r="E19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F19" t="s">
         <v>117</v>
       </c>
-      <c r="B19" t="s">
-        <v>104</v>
-      </c>
-      <c r="C19" t="s">
-        <v>13</v>
-      </c>
-      <c r="D19" t="s">
-        <v>13</v>
-      </c>
-      <c r="E19" t="s">
-        <v>13</v>
-      </c>
-      <c r="F19" t="s">
+      <c r="G19" t="s">
+        <v>15</v>
+      </c>
+      <c r="H19" t="s">
         <v>118</v>
-      </c>
-      <c r="G19" t="s">
-        <v>15</v>
-      </c>
-      <c r="H19" t="s">
-        <v>106</v>
       </c>
       <c r="I19" t="s">
         <v>119</v>
@@ -3100,270 +3115,270 @@
         <v>122</v>
       </c>
       <c r="B20" t="s">
+        <v>109</v>
+      </c>
+      <c r="C20" t="s">
+        <v>13</v>
+      </c>
+      <c r="D20" t="s">
+        <v>13</v>
+      </c>
+      <c r="E20" t="s">
+        <v>13</v>
+      </c>
+      <c r="F20" t="s">
         <v>123</v>
       </c>
-      <c r="C20" t="s">
-        <v>13</v>
-      </c>
-      <c r="D20" t="s">
-        <v>13</v>
-      </c>
-      <c r="E20" t="s">
-        <v>13</v>
-      </c>
-      <c r="F20" t="s">
+      <c r="G20" t="s">
+        <v>15</v>
+      </c>
+      <c r="H20" t="s">
+        <v>111</v>
+      </c>
+      <c r="I20" t="s">
         <v>124</v>
       </c>
-      <c r="G20" t="s">
-        <v>15</v>
-      </c>
-      <c r="H20" t="s">
-        <v>16</v>
-      </c>
-      <c r="I20" t="s">
+      <c r="J20" t="s">
         <v>125</v>
       </c>
-      <c r="J20" t="s">
+      <c r="K20" t="s">
         <v>126</v>
-      </c>
-      <c r="K20" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>127</v>
+      </c>
+      <c r="B21" t="s">
         <v>128</v>
       </c>
-      <c r="B21" t="s">
+      <c r="C21" t="s">
+        <v>13</v>
+      </c>
+      <c r="D21" t="s">
+        <v>13</v>
+      </c>
+      <c r="E21" t="s">
+        <v>13</v>
+      </c>
+      <c r="F21" t="s">
         <v>129</v>
       </c>
-      <c r="C21" t="s">
-        <v>13</v>
-      </c>
-      <c r="D21" t="s">
-        <v>13</v>
-      </c>
-      <c r="E21" t="s">
-        <v>13</v>
-      </c>
-      <c r="F21" t="s">
+      <c r="G21" t="s">
+        <v>15</v>
+      </c>
+      <c r="H21" t="s">
+        <v>16</v>
+      </c>
+      <c r="I21" t="s">
         <v>130</v>
       </c>
-      <c r="G21" t="s">
-        <v>15</v>
-      </c>
-      <c r="H21" t="s">
+      <c r="J21" t="s">
         <v>131</v>
       </c>
-      <c r="I21" t="s">
+      <c r="K21" t="s">
         <v>132</v>
-      </c>
-      <c r="J21" t="s">
-        <v>133</v>
-      </c>
-      <c r="K21" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>133</v>
+      </c>
+      <c r="B22" t="s">
+        <v>134</v>
+      </c>
+      <c r="C22" t="s">
+        <v>13</v>
+      </c>
+      <c r="D22" t="s">
+        <v>13</v>
+      </c>
+      <c r="E22" t="s">
+        <v>13</v>
+      </c>
+      <c r="F22" t="s">
         <v>135</v>
       </c>
-      <c r="B22" t="s">
+      <c r="G22" t="s">
+        <v>15</v>
+      </c>
+      <c r="H22" t="s">
         <v>136</v>
       </c>
-      <c r="C22" t="s">
-        <v>13</v>
-      </c>
-      <c r="D22" t="s">
-        <v>13</v>
-      </c>
-      <c r="E22" t="s">
-        <v>13</v>
-      </c>
-      <c r="F22" t="s">
+      <c r="I22" t="s">
         <v>137</v>
       </c>
-      <c r="G22" t="s">
-        <v>15</v>
-      </c>
-      <c r="H22" t="s">
-        <v>131</v>
-      </c>
-      <c r="I22" t="s">
+      <c r="J22" t="s">
         <v>138</v>
       </c>
-      <c r="J22" t="s">
+      <c r="K22" t="s">
         <v>139</v>
-      </c>
-      <c r="K22" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>140</v>
+      </c>
+      <c r="B23" t="s">
         <v>141</v>
       </c>
-      <c r="B23" t="s">
+      <c r="C23" t="s">
+        <v>13</v>
+      </c>
+      <c r="D23" t="s">
+        <v>13</v>
+      </c>
+      <c r="E23" t="s">
+        <v>13</v>
+      </c>
+      <c r="F23" t="s">
         <v>142</v>
       </c>
-      <c r="C23" t="s">
-        <v>13</v>
-      </c>
-      <c r="D23" t="s">
-        <v>13</v>
-      </c>
-      <c r="E23" t="s">
-        <v>13</v>
-      </c>
-      <c r="F23" t="s">
+      <c r="G23" t="s">
+        <v>15</v>
+      </c>
+      <c r="H23" t="s">
+        <v>136</v>
+      </c>
+      <c r="I23" t="s">
         <v>143</v>
       </c>
-      <c r="G23" t="s">
-        <v>15</v>
-      </c>
-      <c r="H23" t="s">
-        <v>131</v>
-      </c>
-      <c r="I23" t="s">
+      <c r="J23" t="s">
         <v>144</v>
       </c>
-      <c r="J23" t="s">
+      <c r="K23" t="s">
         <v>145</v>
-      </c>
-      <c r="K23" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>146</v>
+      </c>
+      <c r="B24" t="s">
         <v>147</v>
       </c>
-      <c r="B24" t="s">
+      <c r="C24" t="s">
+        <v>13</v>
+      </c>
+      <c r="D24" t="s">
+        <v>13</v>
+      </c>
+      <c r="E24" t="s">
+        <v>13</v>
+      </c>
+      <c r="F24" t="s">
         <v>148</v>
       </c>
-      <c r="C24" t="s">
-        <v>13</v>
-      </c>
-      <c r="D24" t="s">
-        <v>13</v>
-      </c>
-      <c r="E24" t="s">
-        <v>13</v>
-      </c>
-      <c r="F24" t="s">
+      <c r="G24" t="s">
+        <v>15</v>
+      </c>
+      <c r="H24" t="s">
+        <v>136</v>
+      </c>
+      <c r="I24" t="s">
         <v>149</v>
       </c>
-      <c r="G24" t="s">
-        <v>15</v>
-      </c>
-      <c r="H24" t="s">
-        <v>131</v>
-      </c>
-      <c r="I24" t="s">
+      <c r="J24" t="s">
         <v>150</v>
       </c>
-      <c r="J24" t="s">
+      <c r="K24" t="s">
         <v>151</v>
-      </c>
-      <c r="K24" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>152</v>
+      </c>
+      <c r="B25" t="s">
         <v>153</v>
       </c>
-      <c r="B25" t="s">
+      <c r="C25" t="s">
+        <v>13</v>
+      </c>
+      <c r="D25" t="s">
+        <v>13</v>
+      </c>
+      <c r="E25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F25" t="s">
         <v>154</v>
       </c>
-      <c r="C25" t="s">
-        <v>13</v>
-      </c>
-      <c r="D25" t="s">
-        <v>13</v>
-      </c>
-      <c r="E25" t="s">
-        <v>13</v>
-      </c>
-      <c r="F25" t="s">
+      <c r="G25" t="s">
+        <v>15</v>
+      </c>
+      <c r="H25" t="s">
+        <v>136</v>
+      </c>
+      <c r="I25" t="s">
         <v>155</v>
       </c>
-      <c r="G25" t="s">
-        <v>15</v>
-      </c>
-      <c r="H25" t="s">
-        <v>131</v>
-      </c>
-      <c r="I25" t="s">
+      <c r="J25" t="s">
         <v>156</v>
       </c>
-      <c r="J25" t="s">
+      <c r="K25" t="s">
         <v>157</v>
-      </c>
-      <c r="K25" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>158</v>
+      </c>
+      <c r="B26" t="s">
         <v>159</v>
       </c>
-      <c r="B26" t="s">
+      <c r="C26" t="s">
+        <v>13</v>
+      </c>
+      <c r="D26" t="s">
+        <v>13</v>
+      </c>
+      <c r="E26" t="s">
+        <v>13</v>
+      </c>
+      <c r="F26" t="s">
         <v>160</v>
       </c>
-      <c r="C26" t="s">
-        <v>13</v>
-      </c>
-      <c r="D26" t="s">
-        <v>13</v>
-      </c>
-      <c r="E26" t="s">
-        <v>13</v>
-      </c>
-      <c r="F26" t="s">
+      <c r="G26" t="s">
+        <v>15</v>
+      </c>
+      <c r="H26" t="s">
+        <v>136</v>
+      </c>
+      <c r="I26" t="s">
         <v>161</v>
       </c>
-      <c r="G26" t="s">
-        <v>15</v>
-      </c>
-      <c r="H26" t="s">
+      <c r="J26" t="s">
         <v>162</v>
       </c>
-      <c r="I26" t="s">
+      <c r="K26" t="s">
         <v>163</v>
-      </c>
-      <c r="J26" t="s">
-        <v>164</v>
-      </c>
-      <c r="K26" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>164</v>
+      </c>
+      <c r="B27" t="s">
+        <v>165</v>
+      </c>
+      <c r="C27" t="s">
+        <v>13</v>
+      </c>
+      <c r="D27" t="s">
+        <v>13</v>
+      </c>
+      <c r="E27" t="s">
+        <v>13</v>
+      </c>
+      <c r="F27" t="s">
         <v>166</v>
       </c>
-      <c r="B27" t="s">
-        <v>13</v>
-      </c>
-      <c r="C27" t="s">
-        <v>13</v>
-      </c>
-      <c r="D27">
-        <v>2</v>
-      </c>
-      <c r="E27" t="s">
-        <v>13</v>
-      </c>
-      <c r="F27" t="s">
+      <c r="G27" t="s">
+        <v>15</v>
+      </c>
+      <c r="H27" t="s">
         <v>167</v>
-      </c>
-      <c r="G27" t="s">
-        <v>15</v>
-      </c>
-      <c r="H27" t="s">
-        <v>13</v>
       </c>
       <c r="I27" t="s">
         <v>168</v>
@@ -3380,101 +3395,101 @@
         <v>171</v>
       </c>
       <c r="B28" t="s">
+        <v>13</v>
+      </c>
+      <c r="C28" t="s">
+        <v>13</v>
+      </c>
+      <c r="D28">
+        <v>2</v>
+      </c>
+      <c r="E28" t="s">
+        <v>13</v>
+      </c>
+      <c r="F28" t="s">
         <v>172</v>
       </c>
-      <c r="C28" t="s">
-        <v>13</v>
-      </c>
-      <c r="D28" t="s">
-        <v>13</v>
-      </c>
-      <c r="E28" t="s">
-        <v>13</v>
-      </c>
-      <c r="F28" t="s">
+      <c r="G28" t="s">
+        <v>15</v>
+      </c>
+      <c r="H28" t="s">
+        <v>13</v>
+      </c>
+      <c r="I28" t="s">
         <v>173</v>
       </c>
-      <c r="G28" t="s">
-        <v>15</v>
-      </c>
-      <c r="H28" t="s">
+      <c r="J28" t="s">
         <v>174</v>
       </c>
-      <c r="I28" t="s">
+      <c r="K28" t="s">
         <v>175</v>
-      </c>
-      <c r="J28" t="s">
-        <v>176</v>
-      </c>
-      <c r="K28" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>176</v>
+      </c>
+      <c r="B29" t="s">
+        <v>177</v>
+      </c>
+      <c r="C29" t="s">
+        <v>13</v>
+      </c>
+      <c r="D29" t="s">
+        <v>13</v>
+      </c>
+      <c r="E29" t="s">
+        <v>13</v>
+      </c>
+      <c r="F29" t="s">
         <v>178</v>
       </c>
-      <c r="B29" t="s">
-        <v>21</v>
-      </c>
-      <c r="C29" t="s">
-        <v>13</v>
-      </c>
-      <c r="D29" t="s">
-        <v>13</v>
-      </c>
-      <c r="E29" t="s">
-        <v>13</v>
-      </c>
-      <c r="F29" t="s">
+      <c r="G29" t="s">
+        <v>15</v>
+      </c>
+      <c r="H29" t="s">
         <v>179</v>
       </c>
-      <c r="G29" t="s">
-        <v>15</v>
-      </c>
-      <c r="H29" t="s">
+      <c r="I29" t="s">
         <v>180</v>
       </c>
-      <c r="I29" t="s">
+      <c r="J29" t="s">
         <v>181</v>
       </c>
-      <c r="J29" t="s">
+      <c r="K29" t="s">
         <v>182</v>
-      </c>
-      <c r="K29" t="s">
-        <v>183</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>183</v>
+      </c>
+      <c r="B30" t="s">
+        <v>28</v>
+      </c>
+      <c r="C30" t="s">
+        <v>13</v>
+      </c>
+      <c r="D30" t="s">
+        <v>13</v>
+      </c>
+      <c r="E30" t="s">
+        <v>13</v>
+      </c>
+      <c r="F30" t="s">
         <v>184</v>
       </c>
-      <c r="B30" t="s">
-        <v>111</v>
-      </c>
-      <c r="C30" t="s">
-        <v>13</v>
-      </c>
-      <c r="D30" t="s">
-        <v>13</v>
-      </c>
-      <c r="E30" t="s">
-        <v>13</v>
-      </c>
-      <c r="F30" t="s">
+      <c r="G30" t="s">
+        <v>15</v>
+      </c>
+      <c r="H30" t="s">
         <v>185</v>
       </c>
-      <c r="G30" t="s">
-        <v>15</v>
-      </c>
-      <c r="H30" t="s">
+      <c r="I30" t="s">
         <v>186</v>
       </c>
-      <c r="I30" t="s">
+      <c r="J30" t="s">
         <v>187</v>
-      </c>
-      <c r="J30" t="s">
-        <v>13</v>
       </c>
       <c r="K30" t="s">
         <v>188</v>
@@ -3485,7 +3500,7 @@
         <v>189</v>
       </c>
       <c r="B31" t="s">
-        <v>34</v>
+        <v>116</v>
       </c>
       <c r="C31" t="s">
         <v>13</v>
@@ -3509,106 +3524,106 @@
         <v>192</v>
       </c>
       <c r="J31" t="s">
+        <v>13</v>
+      </c>
+      <c r="K31" t="s">
         <v>193</v>
-      </c>
-      <c r="K31" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
+        <v>194</v>
+      </c>
+      <c r="B32" t="s">
+        <v>21</v>
+      </c>
+      <c r="C32" t="s">
+        <v>13</v>
+      </c>
+      <c r="D32" t="s">
+        <v>13</v>
+      </c>
+      <c r="E32" t="s">
+        <v>13</v>
+      </c>
+      <c r="F32" t="s">
         <v>195</v>
       </c>
-      <c r="B32" t="s">
+      <c r="G32" t="s">
+        <v>15</v>
+      </c>
+      <c r="H32" t="s">
         <v>196</v>
       </c>
-      <c r="C32" t="s">
-        <v>13</v>
-      </c>
-      <c r="D32" t="s">
-        <v>13</v>
-      </c>
-      <c r="E32" t="s">
-        <v>13</v>
-      </c>
-      <c r="F32" t="s">
+      <c r="I32" t="s">
         <v>197</v>
       </c>
-      <c r="G32" t="s">
-        <v>15</v>
-      </c>
-      <c r="H32" t="s">
+      <c r="J32" t="s">
         <v>198</v>
       </c>
-      <c r="I32" t="s">
+      <c r="K32" t="s">
         <v>199</v>
-      </c>
-      <c r="J32" t="s">
-        <v>200</v>
-      </c>
-      <c r="K32" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
+        <v>200</v>
+      </c>
+      <c r="B33" t="s">
+        <v>201</v>
+      </c>
+      <c r="C33" t="s">
+        <v>13</v>
+      </c>
+      <c r="D33" t="s">
+        <v>13</v>
+      </c>
+      <c r="E33" t="s">
+        <v>13</v>
+      </c>
+      <c r="F33" t="s">
         <v>202</v>
       </c>
-      <c r="B33" t="s">
+      <c r="G33" t="s">
+        <v>15</v>
+      </c>
+      <c r="H33" t="s">
         <v>203</v>
       </c>
-      <c r="C33" t="s">
-        <v>13</v>
-      </c>
-      <c r="D33" t="s">
-        <v>13</v>
-      </c>
-      <c r="E33" t="s">
-        <v>13</v>
-      </c>
-      <c r="F33" t="s">
+      <c r="I33" t="s">
         <v>204</v>
       </c>
-      <c r="G33" t="s">
-        <v>15</v>
-      </c>
-      <c r="H33" t="s">
+      <c r="J33" t="s">
         <v>205</v>
       </c>
-      <c r="I33" t="s">
+      <c r="K33" t="s">
         <v>206</v>
-      </c>
-      <c r="J33" t="s">
-        <v>207</v>
-      </c>
-      <c r="K33" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
+        <v>207</v>
+      </c>
+      <c r="B34" t="s">
+        <v>208</v>
+      </c>
+      <c r="C34" t="s">
+        <v>13</v>
+      </c>
+      <c r="D34" t="s">
+        <v>13</v>
+      </c>
+      <c r="E34" t="s">
+        <v>13</v>
+      </c>
+      <c r="F34" t="s">
         <v>209</v>
       </c>
-      <c r="B34" t="s">
-        <v>196</v>
-      </c>
-      <c r="C34" t="s">
-        <v>13</v>
-      </c>
-      <c r="D34" t="s">
-        <v>13</v>
-      </c>
-      <c r="E34" t="s">
-        <v>13</v>
-      </c>
-      <c r="F34" t="s">
+      <c r="G34" t="s">
+        <v>15</v>
+      </c>
+      <c r="H34" t="s">
         <v>210</v>
-      </c>
-      <c r="G34" t="s">
-        <v>15</v>
-      </c>
-      <c r="H34" t="s">
-        <v>198</v>
       </c>
       <c r="I34" t="s">
         <v>211</v>
@@ -3625,235 +3640,235 @@
         <v>214</v>
       </c>
       <c r="B35" t="s">
+        <v>201</v>
+      </c>
+      <c r="C35" t="s">
+        <v>13</v>
+      </c>
+      <c r="D35" t="s">
+        <v>13</v>
+      </c>
+      <c r="E35" t="s">
+        <v>13</v>
+      </c>
+      <c r="F35" t="s">
         <v>215</v>
       </c>
-      <c r="C35" t="s">
-        <v>13</v>
-      </c>
-      <c r="D35" t="s">
-        <v>13</v>
-      </c>
-      <c r="E35" t="s">
-        <v>13</v>
-      </c>
-      <c r="F35" t="s">
+      <c r="G35" t="s">
+        <v>15</v>
+      </c>
+      <c r="H35" t="s">
+        <v>203</v>
+      </c>
+      <c r="I35" t="s">
         <v>216</v>
       </c>
-      <c r="G35" t="s">
-        <v>15</v>
-      </c>
-      <c r="H35" t="s">
+      <c r="J35" t="s">
         <v>217</v>
       </c>
-      <c r="I35" t="s">
+      <c r="K35" t="s">
         <v>218</v>
-      </c>
-      <c r="J35" t="s">
-        <v>219</v>
-      </c>
-      <c r="K35" t="s">
-        <v>220</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
+        <v>219</v>
+      </c>
+      <c r="B36" t="s">
+        <v>220</v>
+      </c>
+      <c r="C36" t="s">
+        <v>13</v>
+      </c>
+      <c r="D36" t="s">
+        <v>13</v>
+      </c>
+      <c r="E36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F36" t="s">
         <v>221</v>
       </c>
-      <c r="B36" t="s">
+      <c r="G36" t="s">
+        <v>15</v>
+      </c>
+      <c r="H36" t="s">
         <v>222</v>
       </c>
-      <c r="C36" t="s">
-        <v>13</v>
-      </c>
-      <c r="D36" t="s">
-        <v>13</v>
-      </c>
-      <c r="E36" t="s">
-        <v>13</v>
-      </c>
-      <c r="F36" t="s">
+      <c r="I36" t="s">
         <v>223</v>
       </c>
-      <c r="G36" t="s">
-        <v>15</v>
-      </c>
-      <c r="H36" t="s">
-        <v>82</v>
-      </c>
-      <c r="I36" t="s">
+      <c r="J36" t="s">
         <v>224</v>
       </c>
-      <c r="J36" t="s">
+      <c r="K36" t="s">
         <v>225</v>
-      </c>
-      <c r="K36" t="s">
-        <v>226</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
+        <v>226</v>
+      </c>
+      <c r="B37" t="s">
         <v>227</v>
       </c>
-      <c r="B37" t="s">
+      <c r="C37" t="s">
+        <v>13</v>
+      </c>
+      <c r="D37" t="s">
+        <v>13</v>
+      </c>
+      <c r="E37" t="s">
+        <v>13</v>
+      </c>
+      <c r="F37" t="s">
         <v>228</v>
       </c>
-      <c r="C37" t="s">
-        <v>13</v>
-      </c>
-      <c r="D37" t="s">
-        <v>13</v>
-      </c>
-      <c r="E37" t="s">
-        <v>13</v>
-      </c>
-      <c r="F37" t="s">
+      <c r="G37" t="s">
+        <v>15</v>
+      </c>
+      <c r="H37" t="s">
+        <v>87</v>
+      </c>
+      <c r="I37" t="s">
         <v>229</v>
       </c>
-      <c r="G37" t="s">
-        <v>15</v>
-      </c>
-      <c r="H37" t="s">
+      <c r="J37" t="s">
         <v>230</v>
       </c>
-      <c r="I37" t="s">
+      <c r="K37" t="s">
         <v>231</v>
-      </c>
-      <c r="J37" t="s">
-        <v>232</v>
-      </c>
-      <c r="K37" t="s">
-        <v>233</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
+        <v>232</v>
+      </c>
+      <c r="B38" t="s">
+        <v>233</v>
+      </c>
+      <c r="C38" t="s">
+        <v>13</v>
+      </c>
+      <c r="D38" t="s">
+        <v>13</v>
+      </c>
+      <c r="E38" t="s">
+        <v>13</v>
+      </c>
+      <c r="F38" t="s">
         <v>234</v>
       </c>
-      <c r="B38" t="s">
+      <c r="G38" t="s">
+        <v>15</v>
+      </c>
+      <c r="H38" t="s">
         <v>235</v>
       </c>
-      <c r="C38" t="s">
+      <c r="I38" t="s">
         <v>236</v>
       </c>
-      <c r="D38" t="s">
-        <v>13</v>
-      </c>
-      <c r="E38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F38" t="s">
+      <c r="J38" t="s">
         <v>237</v>
       </c>
-      <c r="G38" t="s">
-        <v>15</v>
-      </c>
-      <c r="H38" t="s">
+      <c r="K38" t="s">
         <v>238</v>
-      </c>
-      <c r="I38" t="s">
-        <v>239</v>
-      </c>
-      <c r="J38" t="s">
-        <v>240</v>
-      </c>
-      <c r="K38" t="s">
-        <v>241</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
+        <v>239</v>
+      </c>
+      <c r="B39" t="s">
+        <v>240</v>
+      </c>
+      <c r="C39" t="s">
+        <v>241</v>
+      </c>
+      <c r="D39" t="s">
+        <v>13</v>
+      </c>
+      <c r="E39" t="s">
+        <v>13</v>
+      </c>
+      <c r="F39" t="s">
         <v>242</v>
       </c>
-      <c r="B39" t="s">
+      <c r="G39" t="s">
+        <v>15</v>
+      </c>
+      <c r="H39" t="s">
         <v>243</v>
       </c>
-      <c r="C39" t="s">
-        <v>13</v>
-      </c>
-      <c r="D39" t="s">
-        <v>13</v>
-      </c>
-      <c r="E39" t="s">
-        <v>13</v>
-      </c>
-      <c r="F39" t="s">
+      <c r="I39" t="s">
         <v>244</v>
       </c>
-      <c r="G39" t="s">
-        <v>15</v>
-      </c>
-      <c r="H39" t="s">
+      <c r="J39" t="s">
         <v>245</v>
       </c>
-      <c r="I39" t="s">
+      <c r="K39" t="s">
         <v>246</v>
-      </c>
-      <c r="J39" t="s">
-        <v>247</v>
-      </c>
-      <c r="K39" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
+        <v>247</v>
+      </c>
+      <c r="B40" t="s">
+        <v>248</v>
+      </c>
+      <c r="C40" t="s">
+        <v>13</v>
+      </c>
+      <c r="D40" t="s">
+        <v>13</v>
+      </c>
+      <c r="E40" t="s">
+        <v>13</v>
+      </c>
+      <c r="F40" t="s">
         <v>249</v>
       </c>
-      <c r="B40" t="s">
+      <c r="G40" t="s">
+        <v>15</v>
+      </c>
+      <c r="H40" t="s">
         <v>250</v>
       </c>
-      <c r="C40" t="s">
-        <v>13</v>
-      </c>
-      <c r="D40" t="s">
-        <v>13</v>
-      </c>
-      <c r="E40" t="s">
-        <v>13</v>
-      </c>
-      <c r="F40" t="s">
+      <c r="I40" t="s">
         <v>251</v>
       </c>
-      <c r="G40" t="s">
-        <v>15</v>
-      </c>
-      <c r="H40" t="s">
+      <c r="J40" t="s">
         <v>252</v>
       </c>
-      <c r="I40" t="s">
+      <c r="K40" t="s">
         <v>253</v>
-      </c>
-      <c r="J40" t="s">
-        <v>254</v>
-      </c>
-      <c r="K40" t="s">
-        <v>255</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
+        <v>254</v>
+      </c>
+      <c r="B41" t="s">
+        <v>255</v>
+      </c>
+      <c r="C41" t="s">
+        <v>13</v>
+      </c>
+      <c r="D41" t="s">
+        <v>13</v>
+      </c>
+      <c r="E41" t="s">
+        <v>13</v>
+      </c>
+      <c r="F41" t="s">
         <v>256</v>
       </c>
-      <c r="B41" t="s">
-        <v>104</v>
-      </c>
-      <c r="C41" t="s">
-        <v>13</v>
-      </c>
-      <c r="D41" t="s">
-        <v>13</v>
-      </c>
-      <c r="E41" t="s">
-        <v>13</v>
-      </c>
-      <c r="F41" t="s">
+      <c r="G41" t="s">
+        <v>15</v>
+      </c>
+      <c r="H41" t="s">
         <v>257</v>
-      </c>
-      <c r="G41" t="s">
-        <v>15</v>
-      </c>
-      <c r="H41" t="s">
-        <v>106</v>
       </c>
       <c r="I41" t="s">
         <v>258</v>
@@ -3870,7 +3885,7 @@
         <v>261</v>
       </c>
       <c r="B42" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="C42" t="s">
         <v>13</v>
@@ -3888,7 +3903,7 @@
         <v>15</v>
       </c>
       <c r="H42" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="I42" t="s">
         <v>263</v>
@@ -3905,7 +3920,7 @@
         <v>266</v>
       </c>
       <c r="B43" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="C43" t="s">
         <v>13</v>
@@ -3923,7 +3938,7 @@
         <v>15</v>
       </c>
       <c r="H43" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="I43" t="s">
         <v>268</v>
@@ -3940,42 +3955,42 @@
         <v>271</v>
       </c>
       <c r="B44" t="s">
+        <v>109</v>
+      </c>
+      <c r="C44" t="s">
+        <v>13</v>
+      </c>
+      <c r="D44" t="s">
+        <v>13</v>
+      </c>
+      <c r="E44" t="s">
+        <v>13</v>
+      </c>
+      <c r="F44" t="s">
         <v>272</v>
       </c>
-      <c r="C44" t="s">
-        <v>13</v>
-      </c>
-      <c r="D44" t="s">
-        <v>13</v>
-      </c>
-      <c r="E44" t="s">
-        <v>13</v>
-      </c>
-      <c r="F44" t="s">
+      <c r="G44" t="s">
+        <v>15</v>
+      </c>
+      <c r="H44" t="s">
+        <v>111</v>
+      </c>
+      <c r="I44" t="s">
         <v>273</v>
       </c>
-      <c r="G44" t="s">
-        <v>15</v>
-      </c>
-      <c r="H44" t="s">
+      <c r="J44" t="s">
         <v>274</v>
       </c>
-      <c r="I44" t="s">
+      <c r="K44" t="s">
         <v>275</v>
-      </c>
-      <c r="J44" t="s">
-        <v>13</v>
-      </c>
-      <c r="K44" t="s">
-        <v>276</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
+        <v>276</v>
+      </c>
+      <c r="B45" t="s">
         <v>277</v>
-      </c>
-      <c r="B45" t="s">
-        <v>104</v>
       </c>
       <c r="C45" t="s">
         <v>13</v>
@@ -3993,13 +4008,13 @@
         <v>15</v>
       </c>
       <c r="H45" t="s">
-        <v>106</v>
+        <v>279</v>
       </c>
       <c r="I45" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="J45" t="s">
-        <v>280</v>
+        <v>13</v>
       </c>
       <c r="K45" t="s">
         <v>281</v>
@@ -4010,7 +4025,7 @@
         <v>282</v>
       </c>
       <c r="B46" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="C46" t="s">
         <v>13</v>
@@ -4028,7 +4043,7 @@
         <v>15</v>
       </c>
       <c r="H46" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="I46" t="s">
         <v>284</v>
@@ -4045,235 +4060,235 @@
         <v>287</v>
       </c>
       <c r="B47" t="s">
+        <v>109</v>
+      </c>
+      <c r="C47" t="s">
+        <v>13</v>
+      </c>
+      <c r="D47" t="s">
+        <v>13</v>
+      </c>
+      <c r="E47" t="s">
+        <v>13</v>
+      </c>
+      <c r="F47" t="s">
         <v>288</v>
       </c>
-      <c r="C47" t="s">
-        <v>13</v>
-      </c>
-      <c r="D47" t="s">
-        <v>13</v>
-      </c>
-      <c r="E47" t="s">
-        <v>13</v>
-      </c>
-      <c r="F47" t="s">
+      <c r="G47" t="s">
+        <v>15</v>
+      </c>
+      <c r="H47" t="s">
+        <v>111</v>
+      </c>
+      <c r="I47" t="s">
         <v>289</v>
       </c>
-      <c r="G47" t="s">
-        <v>15</v>
-      </c>
-      <c r="H47" t="s">
+      <c r="J47" t="s">
         <v>290</v>
       </c>
-      <c r="I47" t="s">
+      <c r="K47" t="s">
         <v>291</v>
-      </c>
-      <c r="J47" t="s">
-        <v>292</v>
-      </c>
-      <c r="K47" t="s">
-        <v>293</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
+        <v>292</v>
+      </c>
+      <c r="B48" t="s">
+        <v>293</v>
+      </c>
+      <c r="C48" t="s">
+        <v>13</v>
+      </c>
+      <c r="D48" t="s">
+        <v>13</v>
+      </c>
+      <c r="E48" t="s">
+        <v>13</v>
+      </c>
+      <c r="F48" t="s">
         <v>294</v>
       </c>
-      <c r="B48" t="s">
+      <c r="G48" t="s">
+        <v>15</v>
+      </c>
+      <c r="H48" t="s">
         <v>295</v>
       </c>
-      <c r="C48" t="s">
-        <v>13</v>
-      </c>
-      <c r="D48" t="s">
-        <v>13</v>
-      </c>
-      <c r="E48" t="s">
-        <v>13</v>
-      </c>
-      <c r="F48" t="s">
+      <c r="I48" t="s">
         <v>296</v>
       </c>
-      <c r="G48" t="s">
-        <v>15</v>
-      </c>
-      <c r="H48" t="s">
+      <c r="J48" t="s">
         <v>297</v>
       </c>
-      <c r="I48" t="s">
+      <c r="K48" t="s">
         <v>298</v>
-      </c>
-      <c r="J48" t="s">
-        <v>299</v>
-      </c>
-      <c r="K48" t="s">
-        <v>300</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
+        <v>299</v>
+      </c>
+      <c r="B49" t="s">
+        <v>300</v>
+      </c>
+      <c r="C49" t="s">
+        <v>13</v>
+      </c>
+      <c r="D49" t="s">
+        <v>13</v>
+      </c>
+      <c r="E49" t="s">
+        <v>13</v>
+      </c>
+      <c r="F49" t="s">
         <v>301</v>
       </c>
-      <c r="B49" t="s">
+      <c r="G49" t="s">
+        <v>15</v>
+      </c>
+      <c r="H49" t="s">
         <v>302</v>
       </c>
-      <c r="C49" t="s">
-        <v>13</v>
-      </c>
-      <c r="D49" t="s">
-        <v>13</v>
-      </c>
-      <c r="E49" t="s">
-        <v>13</v>
-      </c>
-      <c r="F49" t="s">
+      <c r="I49" t="s">
         <v>303</v>
       </c>
-      <c r="G49" t="s">
-        <v>15</v>
-      </c>
-      <c r="H49" t="s">
+      <c r="J49" t="s">
         <v>304</v>
       </c>
-      <c r="I49" t="s">
+      <c r="K49" t="s">
         <v>305</v>
-      </c>
-      <c r="J49" t="s">
-        <v>306</v>
-      </c>
-      <c r="K49" t="s">
-        <v>307</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
+        <v>306</v>
+      </c>
+      <c r="B50" t="s">
+        <v>307</v>
+      </c>
+      <c r="C50" t="s">
+        <v>13</v>
+      </c>
+      <c r="D50" t="s">
+        <v>13</v>
+      </c>
+      <c r="E50" t="s">
+        <v>13</v>
+      </c>
+      <c r="F50" t="s">
         <v>308</v>
       </c>
-      <c r="B50" t="s">
+      <c r="G50" t="s">
+        <v>15</v>
+      </c>
+      <c r="H50" t="s">
         <v>309</v>
       </c>
-      <c r="C50" t="s">
-        <v>13</v>
-      </c>
-      <c r="D50" t="s">
-        <v>13</v>
-      </c>
-      <c r="E50" t="s">
-        <v>13</v>
-      </c>
-      <c r="F50" t="s">
+      <c r="I50" t="s">
         <v>310</v>
       </c>
-      <c r="G50" t="s">
-        <v>15</v>
-      </c>
-      <c r="H50" t="s">
-        <v>297</v>
-      </c>
-      <c r="I50" t="s">
+      <c r="J50" t="s">
         <v>311</v>
       </c>
-      <c r="J50" t="s">
+      <c r="K50" t="s">
         <v>312</v>
-      </c>
-      <c r="K50" t="s">
-        <v>313</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
+        <v>313</v>
+      </c>
+      <c r="B51" t="s">
         <v>314</v>
       </c>
-      <c r="B51" t="s">
+      <c r="C51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51" t="s">
+        <v>13</v>
+      </c>
+      <c r="E51" t="s">
+        <v>13</v>
+      </c>
+      <c r="F51" t="s">
         <v>315</v>
       </c>
-      <c r="C51" t="s">
-        <v>13</v>
-      </c>
-      <c r="D51" t="s">
-        <v>13</v>
-      </c>
-      <c r="E51" t="s">
-        <v>13</v>
-      </c>
-      <c r="F51" t="s">
+      <c r="G51" t="s">
+        <v>15</v>
+      </c>
+      <c r="H51" t="s">
+        <v>302</v>
+      </c>
+      <c r="I51" t="s">
         <v>316</v>
       </c>
-      <c r="G51" t="s">
-        <v>15</v>
-      </c>
-      <c r="H51" t="s">
+      <c r="J51" t="s">
         <v>317</v>
       </c>
-      <c r="I51" t="s">
+      <c r="K51" t="s">
         <v>318</v>
-      </c>
-      <c r="J51" t="s">
-        <v>319</v>
-      </c>
-      <c r="K51" t="s">
-        <v>320</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
+        <v>319</v>
+      </c>
+      <c r="B52" t="s">
+        <v>320</v>
+      </c>
+      <c r="C52" t="s">
+        <v>13</v>
+      </c>
+      <c r="D52" t="s">
+        <v>13</v>
+      </c>
+      <c r="E52" t="s">
+        <v>13</v>
+      </c>
+      <c r="F52" t="s">
         <v>321</v>
       </c>
-      <c r="B52" t="s">
-        <v>104</v>
-      </c>
-      <c r="C52" t="s">
-        <v>13</v>
-      </c>
-      <c r="D52" t="s">
-        <v>13</v>
-      </c>
-      <c r="E52" t="s">
-        <v>13</v>
-      </c>
-      <c r="F52" t="s">
+      <c r="G52" t="s">
+        <v>15</v>
+      </c>
+      <c r="H52" t="s">
         <v>322</v>
       </c>
-      <c r="G52" t="s">
-        <v>15</v>
-      </c>
-      <c r="H52" t="s">
+      <c r="I52" t="s">
         <v>323</v>
       </c>
-      <c r="I52" t="s">
+      <c r="J52" t="s">
         <v>324</v>
       </c>
-      <c r="J52" t="s">
+      <c r="K52" t="s">
         <v>325</v>
-      </c>
-      <c r="K52" t="s">
-        <v>326</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
+        <v>326</v>
+      </c>
+      <c r="B53" t="s">
+        <v>109</v>
+      </c>
+      <c r="C53" t="s">
+        <v>13</v>
+      </c>
+      <c r="D53" t="s">
+        <v>13</v>
+      </c>
+      <c r="E53" t="s">
+        <v>13</v>
+      </c>
+      <c r="F53" t="s">
         <v>327</v>
       </c>
-      <c r="B53" t="s">
-        <v>104</v>
-      </c>
-      <c r="C53" t="s">
-        <v>13</v>
-      </c>
-      <c r="D53" t="s">
-        <v>13</v>
-      </c>
-      <c r="E53" t="s">
-        <v>13</v>
-      </c>
-      <c r="F53" t="s">
+      <c r="G53" t="s">
+        <v>15</v>
+      </c>
+      <c r="H53" t="s">
         <v>328</v>
-      </c>
-      <c r="G53" t="s">
-        <v>15</v>
-      </c>
-      <c r="H53" t="s">
-        <v>323</v>
       </c>
       <c r="I53" t="s">
         <v>329</v>
@@ -4290,112 +4305,112 @@
         <v>332</v>
       </c>
       <c r="B54" t="s">
+        <v>109</v>
+      </c>
+      <c r="C54" t="s">
+        <v>13</v>
+      </c>
+      <c r="D54" t="s">
+        <v>13</v>
+      </c>
+      <c r="E54" t="s">
+        <v>13</v>
+      </c>
+      <c r="F54" t="s">
         <v>333</v>
       </c>
-      <c r="C54" t="s">
-        <v>13</v>
-      </c>
-      <c r="D54" t="s">
-        <v>13</v>
-      </c>
-      <c r="E54" t="s">
-        <v>13</v>
-      </c>
-      <c r="F54" t="s">
+      <c r="G54" t="s">
+        <v>15</v>
+      </c>
+      <c r="H54" t="s">
+        <v>328</v>
+      </c>
+      <c r="I54" t="s">
         <v>334</v>
       </c>
-      <c r="G54" t="s">
-        <v>15</v>
-      </c>
-      <c r="H54" t="s">
-        <v>323</v>
-      </c>
-      <c r="I54" t="s">
+      <c r="J54" t="s">
         <v>335</v>
       </c>
-      <c r="J54" t="s">
+      <c r="K54" t="s">
         <v>336</v>
-      </c>
-      <c r="K54" t="s">
-        <v>337</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
+        <v>337</v>
+      </c>
+      <c r="B55" t="s">
         <v>338</v>
       </c>
-      <c r="B55" t="s">
+      <c r="C55" t="s">
+        <v>13</v>
+      </c>
+      <c r="D55" t="s">
+        <v>13</v>
+      </c>
+      <c r="E55" t="s">
+        <v>13</v>
+      </c>
+      <c r="F55" t="s">
         <v>339</v>
       </c>
-      <c r="C55" t="s">
-        <v>13</v>
-      </c>
-      <c r="D55" t="s">
-        <v>13</v>
-      </c>
-      <c r="E55" t="s">
-        <v>13</v>
-      </c>
-      <c r="F55" t="s">
+      <c r="G55" t="s">
+        <v>15</v>
+      </c>
+      <c r="H55" t="s">
+        <v>328</v>
+      </c>
+      <c r="I55" t="s">
         <v>340</v>
       </c>
-      <c r="G55" t="s">
-        <v>15</v>
-      </c>
-      <c r="H55" t="s">
-        <v>217</v>
-      </c>
-      <c r="I55" t="s">
+      <c r="J55" t="s">
         <v>341</v>
       </c>
-      <c r="J55" t="s">
+      <c r="K55" t="s">
         <v>342</v>
-      </c>
-      <c r="K55" t="s">
-        <v>343</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
+        <v>343</v>
+      </c>
+      <c r="B56" t="s">
         <v>344</v>
       </c>
-      <c r="B56" t="s">
+      <c r="C56" t="s">
+        <v>13</v>
+      </c>
+      <c r="D56" t="s">
+        <v>13</v>
+      </c>
+      <c r="E56" t="s">
+        <v>13</v>
+      </c>
+      <c r="F56" t="s">
         <v>345</v>
       </c>
-      <c r="C56" t="s">
-        <v>13</v>
-      </c>
-      <c r="D56" t="s">
-        <v>13</v>
-      </c>
-      <c r="E56" t="s">
-        <v>13</v>
-      </c>
-      <c r="F56" t="s">
+      <c r="G56" t="s">
+        <v>15</v>
+      </c>
+      <c r="H56" t="s">
+        <v>222</v>
+      </c>
+      <c r="I56" t="s">
         <v>346</v>
       </c>
-      <c r="G56" t="s">
-        <v>15</v>
-      </c>
-      <c r="H56" t="s">
-        <v>230</v>
-      </c>
-      <c r="I56" t="s">
+      <c r="J56" t="s">
         <v>347</v>
       </c>
-      <c r="J56" t="s">
+      <c r="K56" t="s">
         <v>348</v>
-      </c>
-      <c r="K56" t="s">
-        <v>349</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
+        <v>349</v>
+      </c>
+      <c r="B57" t="s">
         <v>350</v>
-      </c>
-      <c r="B57" t="s">
-        <v>345</v>
       </c>
       <c r="C57" t="s">
         <v>13</v>
@@ -4413,7 +4428,7 @@
         <v>15</v>
       </c>
       <c r="H57" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="I57" t="s">
         <v>352</v>
@@ -4430,7 +4445,7 @@
         <v>355</v>
       </c>
       <c r="B58" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
       <c r="C58" t="s">
         <v>13</v>
@@ -4448,7 +4463,7 @@
         <v>15</v>
       </c>
       <c r="H58" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="I58" t="s">
         <v>357</v>
@@ -4465,77 +4480,77 @@
         <v>360</v>
       </c>
       <c r="B59" t="s">
+        <v>350</v>
+      </c>
+      <c r="C59" t="s">
+        <v>13</v>
+      </c>
+      <c r="D59" t="s">
+        <v>13</v>
+      </c>
+      <c r="E59" t="s">
+        <v>13</v>
+      </c>
+      <c r="F59" t="s">
         <v>361</v>
       </c>
-      <c r="C59" t="s">
-        <v>13</v>
-      </c>
-      <c r="D59" t="s">
-        <v>13</v>
-      </c>
-      <c r="E59" t="s">
-        <v>13</v>
-      </c>
-      <c r="F59" t="s">
+      <c r="G59" t="s">
+        <v>15</v>
+      </c>
+      <c r="H59" t="s">
+        <v>235</v>
+      </c>
+      <c r="I59" t="s">
         <v>362</v>
       </c>
-      <c r="G59" t="s">
-        <v>15</v>
-      </c>
-      <c r="H59" t="s">
-        <v>230</v>
-      </c>
-      <c r="I59" t="s">
+      <c r="J59" t="s">
         <v>363</v>
       </c>
-      <c r="J59" t="s">
+      <c r="K59" t="s">
         <v>364</v>
-      </c>
-      <c r="K59" t="s">
-        <v>365</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
+        <v>365</v>
+      </c>
+      <c r="B60" t="s">
         <v>366</v>
       </c>
-      <c r="B60" t="s">
+      <c r="C60" t="s">
+        <v>13</v>
+      </c>
+      <c r="D60" t="s">
+        <v>13</v>
+      </c>
+      <c r="E60" t="s">
+        <v>13</v>
+      </c>
+      <c r="F60" t="s">
         <v>367</v>
       </c>
-      <c r="C60" t="s">
-        <v>13</v>
-      </c>
-      <c r="D60" t="s">
-        <v>13</v>
-      </c>
-      <c r="E60" t="s">
-        <v>13</v>
-      </c>
-      <c r="F60" t="s">
+      <c r="G60" t="s">
+        <v>15</v>
+      </c>
+      <c r="H60" t="s">
+        <v>235</v>
+      </c>
+      <c r="I60" t="s">
         <v>368</v>
       </c>
-      <c r="G60" t="s">
-        <v>15</v>
-      </c>
-      <c r="H60" t="s">
-        <v>230</v>
-      </c>
-      <c r="I60" t="s">
+      <c r="J60" t="s">
         <v>369</v>
       </c>
-      <c r="J60" t="s">
+      <c r="K60" t="s">
         <v>370</v>
-      </c>
-      <c r="K60" t="s">
-        <v>371</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
+        <v>371</v>
+      </c>
+      <c r="B61" t="s">
         <v>372</v>
-      </c>
-      <c r="B61" t="s">
-        <v>345</v>
       </c>
       <c r="C61" t="s">
         <v>13</v>
@@ -4553,7 +4568,7 @@
         <v>15</v>
       </c>
       <c r="H61" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="I61" t="s">
         <v>374</v>
@@ -4570,7 +4585,7 @@
         <v>377</v>
       </c>
       <c r="B62" t="s">
-        <v>104</v>
+        <v>350</v>
       </c>
       <c r="C62" t="s">
         <v>13</v>
@@ -4588,94 +4603,94 @@
         <v>15</v>
       </c>
       <c r="H62" t="s">
+        <v>235</v>
+      </c>
+      <c r="I62" t="s">
         <v>379</v>
       </c>
-      <c r="I62" t="s">
+      <c r="J62" t="s">
         <v>380</v>
       </c>
-      <c r="J62" t="s">
+      <c r="K62" t="s">
         <v>381</v>
-      </c>
-      <c r="K62" t="s">
-        <v>382</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
+        <v>382</v>
+      </c>
+      <c r="B63" t="s">
+        <v>109</v>
+      </c>
+      <c r="C63" t="s">
+        <v>13</v>
+      </c>
+      <c r="D63" t="s">
+        <v>13</v>
+      </c>
+      <c r="E63" t="s">
+        <v>13</v>
+      </c>
+      <c r="F63" t="s">
         <v>383</v>
       </c>
-      <c r="B63" t="s">
+      <c r="G63" t="s">
+        <v>15</v>
+      </c>
+      <c r="H63" t="s">
         <v>384</v>
       </c>
-      <c r="C63" t="s">
-        <v>13</v>
-      </c>
-      <c r="D63" t="s">
-        <v>13</v>
-      </c>
-      <c r="E63" t="s">
-        <v>13</v>
-      </c>
-      <c r="F63" t="s">
+      <c r="I63" t="s">
         <v>385</v>
       </c>
-      <c r="G63" t="s">
-        <v>15</v>
-      </c>
-      <c r="H63" t="s">
-        <v>217</v>
-      </c>
-      <c r="I63" t="s">
+      <c r="J63" t="s">
         <v>386</v>
       </c>
-      <c r="J63" t="s">
+      <c r="K63" t="s">
         <v>387</v>
-      </c>
-      <c r="K63" t="s">
-        <v>388</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
+        <v>388</v>
+      </c>
+      <c r="B64" t="s">
         <v>389</v>
       </c>
-      <c r="B64" t="s">
+      <c r="C64" t="s">
+        <v>13</v>
+      </c>
+      <c r="D64" t="s">
+        <v>13</v>
+      </c>
+      <c r="E64" t="s">
+        <v>13</v>
+      </c>
+      <c r="F64" t="s">
         <v>390</v>
       </c>
-      <c r="C64" t="s">
-        <v>13</v>
-      </c>
-      <c r="D64" t="s">
-        <v>13</v>
-      </c>
-      <c r="E64" t="s">
-        <v>13</v>
-      </c>
-      <c r="F64" t="s">
+      <c r="G64" t="s">
+        <v>15</v>
+      </c>
+      <c r="H64" t="s">
+        <v>222</v>
+      </c>
+      <c r="I64" t="s">
         <v>391</v>
       </c>
-      <c r="G64" t="s">
-        <v>15</v>
-      </c>
-      <c r="H64" t="s">
-        <v>217</v>
-      </c>
-      <c r="I64" t="s">
+      <c r="J64" t="s">
         <v>392</v>
       </c>
-      <c r="J64" t="s">
+      <c r="K64" t="s">
         <v>393</v>
-      </c>
-      <c r="K64" t="s">
-        <v>394</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
+        <v>394</v>
+      </c>
+      <c r="B65" t="s">
         <v>395</v>
-      </c>
-      <c r="B65" t="s">
-        <v>384</v>
       </c>
       <c r="C65" t="s">
         <v>13</v>
@@ -4693,7 +4708,7 @@
         <v>15</v>
       </c>
       <c r="H65" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="I65" t="s">
         <v>397</v>
@@ -4710,7 +4725,7 @@
         <v>400</v>
       </c>
       <c r="B66" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="C66" t="s">
         <v>13</v>
@@ -4728,7 +4743,7 @@
         <v>15</v>
       </c>
       <c r="H66" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="I66" t="s">
         <v>402</v>
@@ -4745,182 +4760,182 @@
         <v>405</v>
       </c>
       <c r="B67" t="s">
-        <v>34</v>
+        <v>395</v>
       </c>
       <c r="C67" t="s">
+        <v>13</v>
+      </c>
+      <c r="D67" t="s">
+        <v>13</v>
+      </c>
+      <c r="E67" t="s">
+        <v>13</v>
+      </c>
+      <c r="F67" t="s">
         <v>406</v>
       </c>
-      <c r="D67" t="s">
-        <v>13</v>
-      </c>
-      <c r="E67" t="s">
-        <v>13</v>
-      </c>
-      <c r="F67" t="s">
+      <c r="G67" t="s">
+        <v>15</v>
+      </c>
+      <c r="H67" t="s">
+        <v>222</v>
+      </c>
+      <c r="I67" t="s">
         <v>407</v>
       </c>
-      <c r="G67" t="s">
-        <v>15</v>
-      </c>
-      <c r="H67" t="s">
+      <c r="J67" t="s">
         <v>408</v>
       </c>
-      <c r="I67" t="s">
+      <c r="K67" t="s">
         <v>409</v>
-      </c>
-      <c r="J67" t="s">
-        <v>410</v>
-      </c>
-      <c r="K67" t="s">
-        <v>411</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
+        <v>410</v>
+      </c>
+      <c r="B68" t="s">
+        <v>21</v>
+      </c>
+      <c r="C68" t="s">
+        <v>411</v>
+      </c>
+      <c r="D68" t="s">
+        <v>13</v>
+      </c>
+      <c r="E68" t="s">
+        <v>13</v>
+      </c>
+      <c r="F68" t="s">
         <v>412</v>
       </c>
-      <c r="B68" t="s">
-        <v>34</v>
-      </c>
-      <c r="C68" t="s">
+      <c r="G68" t="s">
+        <v>15</v>
+      </c>
+      <c r="H68" t="s">
         <v>413</v>
       </c>
-      <c r="D68" t="s">
-        <v>13</v>
-      </c>
-      <c r="E68" t="s">
-        <v>13</v>
-      </c>
-      <c r="F68" t="s">
+      <c r="I68" t="s">
         <v>414</v>
       </c>
-      <c r="G68" t="s">
-        <v>15</v>
-      </c>
-      <c r="H68" t="s">
-        <v>408</v>
-      </c>
-      <c r="I68" t="s">
+      <c r="J68" t="s">
         <v>415</v>
       </c>
-      <c r="J68" t="s">
+      <c r="K68" t="s">
         <v>416</v>
-      </c>
-      <c r="K68" t="s">
-        <v>417</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
+        <v>417</v>
+      </c>
+      <c r="B69" t="s">
+        <v>21</v>
+      </c>
+      <c r="C69" t="s">
         <v>418</v>
       </c>
-      <c r="B69" t="s">
-        <v>34</v>
-      </c>
-      <c r="C69" t="s">
+      <c r="D69" t="s">
+        <v>13</v>
+      </c>
+      <c r="E69" t="s">
+        <v>13</v>
+      </c>
+      <c r="F69" t="s">
         <v>419</v>
       </c>
-      <c r="D69" t="s">
-        <v>13</v>
-      </c>
-      <c r="E69" t="s">
+      <c r="G69" t="s">
+        <v>15</v>
+      </c>
+      <c r="H69" t="s">
+        <v>413</v>
+      </c>
+      <c r="I69" t="s">
         <v>420</v>
       </c>
-      <c r="F69" t="s">
+      <c r="J69" t="s">
         <v>421</v>
       </c>
-      <c r="G69" t="s">
-        <v>15</v>
-      </c>
-      <c r="H69" t="s">
+      <c r="K69" t="s">
         <v>422</v>
-      </c>
-      <c r="I69" t="s">
-        <v>423</v>
-      </c>
-      <c r="J69" t="s">
-        <v>424</v>
-      </c>
-      <c r="K69" t="s">
-        <v>425</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
+        <v>423</v>
+      </c>
+      <c r="B70" t="s">
+        <v>21</v>
+      </c>
+      <c r="C70" t="s">
+        <v>424</v>
+      </c>
+      <c r="D70" t="s">
+        <v>13</v>
+      </c>
+      <c r="E70" t="s">
+        <v>425</v>
+      </c>
+      <c r="F70" t="s">
         <v>426</v>
       </c>
-      <c r="B70" t="s">
+      <c r="G70" t="s">
+        <v>15</v>
+      </c>
+      <c r="H70" t="s">
         <v>427</v>
       </c>
-      <c r="C70" t="s">
-        <v>13</v>
-      </c>
-      <c r="D70" t="s">
-        <v>13</v>
-      </c>
-      <c r="E70" t="s">
-        <v>13</v>
-      </c>
-      <c r="F70" t="s">
+      <c r="I70" t="s">
         <v>428</v>
       </c>
-      <c r="G70" t="s">
-        <v>15</v>
-      </c>
-      <c r="H70" t="s">
+      <c r="J70" t="s">
         <v>429</v>
       </c>
-      <c r="I70" t="s">
+      <c r="K70" t="s">
         <v>430</v>
-      </c>
-      <c r="J70" t="s">
-        <v>431</v>
-      </c>
-      <c r="K70" t="s">
-        <v>432</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
+        <v>431</v>
+      </c>
+      <c r="B71" t="s">
+        <v>432</v>
+      </c>
+      <c r="C71" t="s">
+        <v>13</v>
+      </c>
+      <c r="D71" t="s">
+        <v>13</v>
+      </c>
+      <c r="E71" t="s">
+        <v>13</v>
+      </c>
+      <c r="F71" t="s">
         <v>433</v>
       </c>
-      <c r="B71" t="s">
+      <c r="G71" t="s">
+        <v>15</v>
+      </c>
+      <c r="H71" t="s">
         <v>434</v>
       </c>
-      <c r="C71" t="s">
-        <v>13</v>
-      </c>
-      <c r="D71" t="s">
-        <v>13</v>
-      </c>
-      <c r="E71" t="s">
-        <v>13</v>
-      </c>
-      <c r="F71" t="s">
+      <c r="I71" t="s">
         <v>435</v>
       </c>
-      <c r="G71" t="s">
-        <v>15</v>
-      </c>
-      <c r="H71" t="s">
-        <v>429</v>
-      </c>
-      <c r="I71" t="s">
+      <c r="J71" t="s">
         <v>436</v>
       </c>
-      <c r="J71" t="s">
+      <c r="K71" t="s">
         <v>437</v>
-      </c>
-      <c r="K71" t="s">
-        <v>438</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
+        <v>438</v>
+      </c>
+      <c r="B72" t="s">
         <v>439</v>
-      </c>
-      <c r="B72" t="s">
-        <v>434</v>
       </c>
       <c r="C72" t="s">
         <v>13</v>
@@ -4938,7 +4953,7 @@
         <v>15</v>
       </c>
       <c r="H72" t="s">
-        <v>429</v>
+        <v>434</v>
       </c>
       <c r="I72" t="s">
         <v>441</v>
@@ -4955,7 +4970,7 @@
         <v>444</v>
       </c>
       <c r="B73" t="s">
-        <v>434</v>
+        <v>439</v>
       </c>
       <c r="C73" t="s">
         <v>13</v>
@@ -4973,7 +4988,7 @@
         <v>15</v>
       </c>
       <c r="H73" t="s">
-        <v>429</v>
+        <v>434</v>
       </c>
       <c r="I73" t="s">
         <v>446</v>
@@ -4990,95 +5005,95 @@
         <v>449</v>
       </c>
       <c r="B74" t="s">
+        <v>439</v>
+      </c>
+      <c r="C74" t="s">
+        <v>13</v>
+      </c>
+      <c r="D74" t="s">
+        <v>13</v>
+      </c>
+      <c r="E74" t="s">
+        <v>13</v>
+      </c>
+      <c r="F74" t="s">
         <v>450</v>
       </c>
-      <c r="C74" t="s">
-        <v>13</v>
-      </c>
-      <c r="D74" t="s">
-        <v>13</v>
-      </c>
-      <c r="E74" t="s">
-        <v>13</v>
-      </c>
-      <c r="F74" t="s">
+      <c r="G74" t="s">
+        <v>15</v>
+      </c>
+      <c r="H74" t="s">
+        <v>434</v>
+      </c>
+      <c r="I74" t="s">
         <v>451</v>
       </c>
-      <c r="G74" t="s">
-        <v>15</v>
-      </c>
-      <c r="H74" t="s">
-        <v>429</v>
-      </c>
-      <c r="I74" t="s">
+      <c r="J74" t="s">
         <v>452</v>
       </c>
-      <c r="J74" t="s">
+      <c r="K74" t="s">
         <v>453</v>
-      </c>
-      <c r="K74" t="s">
-        <v>454</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
+        <v>454</v>
+      </c>
+      <c r="B75" t="s">
         <v>455</v>
       </c>
-      <c r="B75" t="s">
+      <c r="C75" t="s">
+        <v>13</v>
+      </c>
+      <c r="D75" t="s">
+        <v>13</v>
+      </c>
+      <c r="E75" t="s">
+        <v>13</v>
+      </c>
+      <c r="F75" t="s">
         <v>456</v>
       </c>
-      <c r="C75" t="s">
-        <v>13</v>
-      </c>
-      <c r="D75" t="s">
-        <v>13</v>
-      </c>
-      <c r="E75" t="s">
-        <v>13</v>
-      </c>
-      <c r="F75" t="s">
+      <c r="G75" t="s">
+        <v>15</v>
+      </c>
+      <c r="H75" t="s">
+        <v>434</v>
+      </c>
+      <c r="I75" t="s">
         <v>457</v>
       </c>
-      <c r="G75" t="s">
-        <v>15</v>
-      </c>
-      <c r="H75" t="s">
+      <c r="J75" t="s">
         <v>458</v>
       </c>
-      <c r="I75" t="s">
+      <c r="K75" t="s">
         <v>459</v>
-      </c>
-      <c r="J75" t="s">
-        <v>460</v>
-      </c>
-      <c r="K75" t="s">
-        <v>461</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
+        <v>460</v>
+      </c>
+      <c r="B76" t="s">
+        <v>461</v>
+      </c>
+      <c r="C76" t="s">
+        <v>13</v>
+      </c>
+      <c r="D76" t="s">
+        <v>13</v>
+      </c>
+      <c r="E76" t="s">
+        <v>13</v>
+      </c>
+      <c r="F76" t="s">
         <v>462</v>
       </c>
-      <c r="B76" t="s">
-        <v>456</v>
-      </c>
-      <c r="C76" t="s">
-        <v>13</v>
-      </c>
-      <c r="D76" t="s">
-        <v>13</v>
-      </c>
-      <c r="E76" t="s">
-        <v>13</v>
-      </c>
-      <c r="F76" t="s">
+      <c r="G76" t="s">
+        <v>15</v>
+      </c>
+      <c r="H76" t="s">
         <v>463</v>
-      </c>
-      <c r="G76" t="s">
-        <v>15</v>
-      </c>
-      <c r="H76" t="s">
-        <v>458</v>
       </c>
       <c r="I76" t="s">
         <v>464</v>
@@ -5095,7 +5110,7 @@
         <v>467</v>
       </c>
       <c r="B77" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
       <c r="C77" t="s">
         <v>13</v>
@@ -5113,7 +5128,7 @@
         <v>15</v>
       </c>
       <c r="H77" t="s">
-        <v>458</v>
+        <v>463</v>
       </c>
       <c r="I77" t="s">
         <v>469</v>
@@ -5130,7 +5145,7 @@
         <v>472</v>
       </c>
       <c r="B78" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
       <c r="C78" t="s">
         <v>13</v>
@@ -5148,7 +5163,7 @@
         <v>15</v>
       </c>
       <c r="H78" t="s">
-        <v>458</v>
+        <v>463</v>
       </c>
       <c r="I78" t="s">
         <v>474</v>
@@ -5157,15 +5172,15 @@
         <v>475</v>
       </c>
       <c r="K78" t="s">
-        <v>170</v>
+        <v>476</v>
       </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="B79" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
       <c r="C79" t="s">
         <v>13</v>
@@ -5177,30 +5192,30 @@
         <v>13</v>
       </c>
       <c r="F79" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="G79" t="s">
         <v>15</v>
       </c>
       <c r="H79" t="s">
-        <v>458</v>
+        <v>463</v>
       </c>
       <c r="I79" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="J79" t="s">
-        <v>13</v>
+        <v>480</v>
       </c>
       <c r="K79" t="s">
-        <v>479</v>
+        <v>175</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="B80" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
       <c r="C80" t="s">
         <v>13</v>
@@ -5212,30 +5227,30 @@
         <v>13</v>
       </c>
       <c r="F80" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="G80" t="s">
         <v>15</v>
       </c>
       <c r="H80" t="s">
-        <v>458</v>
+        <v>463</v>
       </c>
       <c r="I80" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="J80" t="s">
         <v>13</v>
       </c>
       <c r="K80" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="B81" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
       <c r="C81" t="s">
         <v>13</v>
@@ -5247,30 +5262,30 @@
         <v>13</v>
       </c>
       <c r="F81" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="G81" t="s">
         <v>15</v>
       </c>
       <c r="H81" t="s">
-        <v>458</v>
+        <v>463</v>
       </c>
       <c r="I81" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="J81" t="s">
         <v>13</v>
       </c>
       <c r="K81" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="B82" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
       <c r="C82" t="s">
         <v>13</v>
@@ -5282,19 +5297,19 @@
         <v>13</v>
       </c>
       <c r="F82" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="G82" t="s">
         <v>15</v>
       </c>
       <c r="H82" t="s">
-        <v>458</v>
+        <v>463</v>
       </c>
       <c r="I82" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="J82" t="s">
-        <v>491</v>
+        <v>13</v>
       </c>
       <c r="K82" t="s">
         <v>492</v>
@@ -5305,7 +5320,7 @@
         <v>493</v>
       </c>
       <c r="B83" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
       <c r="C83" t="s">
         <v>13</v>
@@ -5323,7 +5338,7 @@
         <v>15</v>
       </c>
       <c r="H83" t="s">
-        <v>458</v>
+        <v>463</v>
       </c>
       <c r="I83" t="s">
         <v>495</v>
@@ -5340,7 +5355,7 @@
         <v>498</v>
       </c>
       <c r="B84" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
       <c r="C84" t="s">
         <v>13</v>
@@ -5358,24 +5373,24 @@
         <v>15</v>
       </c>
       <c r="H84" t="s">
-        <v>458</v>
+        <v>463</v>
       </c>
       <c r="I84" t="s">
         <v>500</v>
       </c>
       <c r="J84" t="s">
-        <v>13</v>
+        <v>501</v>
       </c>
       <c r="K84" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="B85" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
       <c r="C85" t="s">
         <v>13</v>
@@ -5387,19 +5402,19 @@
         <v>13</v>
       </c>
       <c r="F85" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="G85" t="s">
         <v>15</v>
       </c>
       <c r="H85" t="s">
-        <v>458</v>
+        <v>463</v>
       </c>
       <c r="I85" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="J85" t="s">
-        <v>505</v>
+        <v>13</v>
       </c>
       <c r="K85" t="s">
         <v>506</v>
@@ -5410,7 +5425,7 @@
         <v>507</v>
       </c>
       <c r="B86" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
       <c r="C86" t="s">
         <v>13</v>
@@ -5428,7 +5443,7 @@
         <v>15</v>
       </c>
       <c r="H86" t="s">
-        <v>458</v>
+        <v>463</v>
       </c>
       <c r="I86" t="s">
         <v>509</v>
@@ -5445,7 +5460,7 @@
         <v>512</v>
       </c>
       <c r="B87" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
       <c r="C87" t="s">
         <v>13</v>
@@ -5463,24 +5478,24 @@
         <v>15</v>
       </c>
       <c r="H87" t="s">
-        <v>458</v>
+        <v>463</v>
       </c>
       <c r="I87" t="s">
         <v>514</v>
       </c>
       <c r="J87" t="s">
-        <v>13</v>
+        <v>515</v>
       </c>
       <c r="K87" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
     </row>
     <row r="88" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="B88" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
       <c r="C88" t="s">
         <v>13</v>
@@ -5492,19 +5507,19 @@
         <v>13</v>
       </c>
       <c r="F88" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="G88" t="s">
         <v>15</v>
       </c>
       <c r="H88" t="s">
-        <v>458</v>
+        <v>463</v>
       </c>
       <c r="I88" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="J88" t="s">
-        <v>519</v>
+        <v>13</v>
       </c>
       <c r="K88" t="s">
         <v>520</v>
@@ -5515,7 +5530,7 @@
         <v>521</v>
       </c>
       <c r="B89" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
       <c r="C89" t="s">
         <v>13</v>
@@ -5533,7 +5548,7 @@
         <v>15</v>
       </c>
       <c r="H89" t="s">
-        <v>458</v>
+        <v>463</v>
       </c>
       <c r="I89" t="s">
         <v>523</v>
@@ -5550,7 +5565,7 @@
         <v>526</v>
       </c>
       <c r="B90" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
       <c r="C90" t="s">
         <v>13</v>
@@ -5568,24 +5583,24 @@
         <v>15</v>
       </c>
       <c r="H90" t="s">
-        <v>458</v>
+        <v>463</v>
       </c>
       <c r="I90" t="s">
         <v>528</v>
       </c>
       <c r="J90" t="s">
-        <v>13</v>
+        <v>529</v>
       </c>
       <c r="K90" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
     </row>
     <row r="91" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="B91" t="s">
-        <v>104</v>
+        <v>461</v>
       </c>
       <c r="C91" t="s">
         <v>13</v>
@@ -5597,118 +5612,118 @@
         <v>13</v>
       </c>
       <c r="F91" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="G91" t="s">
         <v>15</v>
       </c>
       <c r="H91" t="s">
-        <v>532</v>
+        <v>463</v>
       </c>
       <c r="I91" t="s">
         <v>533</v>
       </c>
       <c r="J91" t="s">
+        <v>13</v>
+      </c>
+      <c r="K91" t="s">
         <v>534</v>
-      </c>
-      <c r="K91" t="s">
-        <v>535</v>
       </c>
     </row>
     <row r="92" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
+        <v>535</v>
+      </c>
+      <c r="B92" t="s">
+        <v>109</v>
+      </c>
+      <c r="C92" t="s">
+        <v>13</v>
+      </c>
+      <c r="D92" t="s">
+        <v>13</v>
+      </c>
+      <c r="E92" t="s">
+        <v>13</v>
+      </c>
+      <c r="F92" t="s">
         <v>536</v>
       </c>
-      <c r="B92" t="s">
+      <c r="G92" t="s">
+        <v>15</v>
+      </c>
+      <c r="H92" t="s">
         <v>537</v>
       </c>
-      <c r="C92" t="s">
-        <v>13</v>
-      </c>
-      <c r="D92" t="s">
-        <v>13</v>
-      </c>
-      <c r="E92" t="s">
-        <v>13</v>
-      </c>
-      <c r="F92" t="s">
+      <c r="I92" t="s">
         <v>538</v>
       </c>
-      <c r="G92" t="s">
-        <v>15</v>
-      </c>
-      <c r="H92" t="s">
-        <v>323</v>
-      </c>
-      <c r="I92" t="s">
+      <c r="J92" t="s">
         <v>539</v>
       </c>
-      <c r="J92" t="s">
+      <c r="K92" t="s">
         <v>540</v>
-      </c>
-      <c r="K92" t="s">
-        <v>541</v>
       </c>
     </row>
     <row r="93" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
+        <v>541</v>
+      </c>
+      <c r="B93" t="s">
         <v>542</v>
       </c>
-      <c r="B93" t="s">
+      <c r="C93" t="s">
+        <v>13</v>
+      </c>
+      <c r="D93" t="s">
+        <v>13</v>
+      </c>
+      <c r="E93" t="s">
+        <v>13</v>
+      </c>
+      <c r="F93" t="s">
         <v>543</v>
       </c>
-      <c r="C93" t="s">
-        <v>13</v>
-      </c>
-      <c r="D93" t="s">
-        <v>13</v>
-      </c>
-      <c r="E93" t="s">
-        <v>13</v>
-      </c>
-      <c r="F93" t="s">
+      <c r="G93" t="s">
+        <v>15</v>
+      </c>
+      <c r="H93" t="s">
+        <v>328</v>
+      </c>
+      <c r="I93" t="s">
         <v>544</v>
       </c>
-      <c r="G93" t="s">
-        <v>15</v>
-      </c>
-      <c r="H93" t="s">
+      <c r="J93" t="s">
         <v>545</v>
       </c>
-      <c r="I93" t="s">
+      <c r="K93" t="s">
         <v>546</v>
-      </c>
-      <c r="J93" t="s">
-        <v>547</v>
-      </c>
-      <c r="K93" t="s">
-        <v>548</v>
       </c>
     </row>
     <row r="94" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
+        <v>547</v>
+      </c>
+      <c r="B94" t="s">
+        <v>548</v>
+      </c>
+      <c r="C94" t="s">
+        <v>13</v>
+      </c>
+      <c r="D94" t="s">
+        <v>13</v>
+      </c>
+      <c r="E94" t="s">
+        <v>13</v>
+      </c>
+      <c r="F94" t="s">
         <v>549</v>
       </c>
-      <c r="B94" t="s">
-        <v>333</v>
-      </c>
-      <c r="C94" t="s">
-        <v>13</v>
-      </c>
-      <c r="D94" t="s">
-        <v>13</v>
-      </c>
-      <c r="E94" t="s">
-        <v>13</v>
-      </c>
-      <c r="F94" t="s">
+      <c r="G94" t="s">
+        <v>15</v>
+      </c>
+      <c r="H94" t="s">
         <v>550</v>
-      </c>
-      <c r="G94" t="s">
-        <v>15</v>
-      </c>
-      <c r="H94" t="s">
-        <v>323</v>
       </c>
       <c r="I94" t="s">
         <v>551</v>
@@ -5725,42 +5740,42 @@
         <v>554</v>
       </c>
       <c r="B95" t="s">
+        <v>338</v>
+      </c>
+      <c r="C95" t="s">
+        <v>13</v>
+      </c>
+      <c r="D95" t="s">
+        <v>13</v>
+      </c>
+      <c r="E95" t="s">
+        <v>13</v>
+      </c>
+      <c r="F95" t="s">
         <v>555</v>
       </c>
-      <c r="C95" t="s">
-        <v>13</v>
-      </c>
-      <c r="D95" t="s">
-        <v>13</v>
-      </c>
-      <c r="E95" t="s">
-        <v>13</v>
-      </c>
-      <c r="F95" t="s">
+      <c r="G95" t="s">
+        <v>15</v>
+      </c>
+      <c r="H95" t="s">
+        <v>328</v>
+      </c>
+      <c r="I95" t="s">
         <v>556</v>
       </c>
-      <c r="G95" t="s">
-        <v>15</v>
-      </c>
-      <c r="H95" t="s">
-        <v>323</v>
-      </c>
-      <c r="I95" t="s">
+      <c r="J95" t="s">
         <v>557</v>
       </c>
-      <c r="J95" t="s">
+      <c r="K95" t="s">
         <v>558</v>
-      </c>
-      <c r="K95" t="s">
-        <v>559</v>
       </c>
     </row>
     <row r="96" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
+        <v>559</v>
+      </c>
+      <c r="B96" t="s">
         <v>560</v>
-      </c>
-      <c r="B96" t="s">
-        <v>537</v>
       </c>
       <c r="C96" t="s">
         <v>13</v>
@@ -5778,7 +5793,7 @@
         <v>15</v>
       </c>
       <c r="H96" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="I96" t="s">
         <v>562</v>
@@ -5795,7 +5810,7 @@
         <v>565</v>
       </c>
       <c r="B97" t="s">
-        <v>104</v>
+        <v>542</v>
       </c>
       <c r="C97" t="s">
         <v>13</v>
@@ -5813,7 +5828,7 @@
         <v>15</v>
       </c>
       <c r="H97" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="I97" t="s">
         <v>567</v>
@@ -5830,7 +5845,7 @@
         <v>570</v>
       </c>
       <c r="B98" t="s">
-        <v>543</v>
+        <v>109</v>
       </c>
       <c r="C98" t="s">
         <v>13</v>
@@ -5848,7 +5863,7 @@
         <v>15</v>
       </c>
       <c r="H98" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="I98" t="s">
         <v>572</v>
@@ -5865,42 +5880,42 @@
         <v>575</v>
       </c>
       <c r="B99" t="s">
+        <v>548</v>
+      </c>
+      <c r="C99" t="s">
+        <v>13</v>
+      </c>
+      <c r="D99" t="s">
+        <v>13</v>
+      </c>
+      <c r="E99" t="s">
+        <v>13</v>
+      </c>
+      <c r="F99" t="s">
         <v>576</v>
       </c>
-      <c r="C99" t="s">
-        <v>13</v>
-      </c>
-      <c r="D99" t="s">
-        <v>13</v>
-      </c>
-      <c r="E99" t="s">
-        <v>13</v>
-      </c>
-      <c r="F99" t="s">
+      <c r="G99" t="s">
+        <v>15</v>
+      </c>
+      <c r="H99" t="s">
+        <v>328</v>
+      </c>
+      <c r="I99" t="s">
         <v>577</v>
       </c>
-      <c r="G99" t="s">
-        <v>15</v>
-      </c>
-      <c r="H99" t="s">
-        <v>545</v>
-      </c>
-      <c r="I99" t="s">
+      <c r="J99" t="s">
         <v>578</v>
       </c>
-      <c r="J99" t="s">
+      <c r="K99" t="s">
         <v>579</v>
-      </c>
-      <c r="K99" t="s">
-        <v>580</v>
       </c>
     </row>
     <row r="100" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
+        <v>580</v>
+      </c>
+      <c r="B100" t="s">
         <v>581</v>
-      </c>
-      <c r="B100" t="s">
-        <v>543</v>
       </c>
       <c r="C100" t="s">
         <v>13</v>
@@ -5918,7 +5933,7 @@
         <v>15</v>
       </c>
       <c r="H100" t="s">
-        <v>323</v>
+        <v>550</v>
       </c>
       <c r="I100" t="s">
         <v>583</v>
@@ -5935,7 +5950,7 @@
         <v>586</v>
       </c>
       <c r="B101" t="s">
-        <v>537</v>
+        <v>548</v>
       </c>
       <c r="C101" t="s">
         <v>13</v>
@@ -5953,7 +5968,7 @@
         <v>15</v>
       </c>
       <c r="H101" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="I101" t="s">
         <v>588</v>
@@ -5970,42 +5985,42 @@
         <v>591</v>
       </c>
       <c r="B102" t="s">
+        <v>542</v>
+      </c>
+      <c r="C102" t="s">
+        <v>13</v>
+      </c>
+      <c r="D102" t="s">
+        <v>13</v>
+      </c>
+      <c r="E102" t="s">
+        <v>13</v>
+      </c>
+      <c r="F102" t="s">
         <v>592</v>
       </c>
-      <c r="C102" t="s">
-        <v>13</v>
-      </c>
-      <c r="D102" t="s">
-        <v>13</v>
-      </c>
-      <c r="E102" t="s">
-        <v>13</v>
-      </c>
-      <c r="F102" t="s">
+      <c r="G102" t="s">
+        <v>15</v>
+      </c>
+      <c r="H102" t="s">
+        <v>328</v>
+      </c>
+      <c r="I102" t="s">
         <v>593</v>
       </c>
-      <c r="G102" t="s">
-        <v>15</v>
-      </c>
-      <c r="H102" t="s">
-        <v>323</v>
-      </c>
-      <c r="I102" t="s">
+      <c r="J102" t="s">
         <v>594</v>
       </c>
-      <c r="J102" t="s">
+      <c r="K102" t="s">
         <v>595</v>
-      </c>
-      <c r="K102" t="s">
-        <v>596</v>
       </c>
     </row>
     <row r="103" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
+        <v>596</v>
+      </c>
+      <c r="B103" t="s">
         <v>597</v>
-      </c>
-      <c r="B103" t="s">
-        <v>543</v>
       </c>
       <c r="C103" t="s">
         <v>13</v>
@@ -6023,7 +6038,7 @@
         <v>15</v>
       </c>
       <c r="H103" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="I103" t="s">
         <v>599</v>
@@ -6040,7 +6055,7 @@
         <v>602</v>
       </c>
       <c r="B104" t="s">
-        <v>537</v>
+        <v>548</v>
       </c>
       <c r="C104" t="s">
         <v>13</v>
@@ -6058,42 +6073,42 @@
         <v>15</v>
       </c>
       <c r="H104" t="s">
+        <v>328</v>
+      </c>
+      <c r="I104" t="s">
         <v>604</v>
       </c>
-      <c r="I104" t="s">
+      <c r="J104" t="s">
         <v>605</v>
       </c>
-      <c r="J104" t="s">
+      <c r="K104" t="s">
         <v>606</v>
-      </c>
-      <c r="K104" t="s">
-        <v>607</v>
       </c>
     </row>
     <row r="105" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
+        <v>607</v>
+      </c>
+      <c r="B105" t="s">
+        <v>542</v>
+      </c>
+      <c r="C105" t="s">
+        <v>13</v>
+      </c>
+      <c r="D105" t="s">
+        <v>13</v>
+      </c>
+      <c r="E105" t="s">
+        <v>13</v>
+      </c>
+      <c r="F105" t="s">
         <v>608</v>
       </c>
-      <c r="B105" t="s">
-        <v>543</v>
-      </c>
-      <c r="C105" t="s">
-        <v>13</v>
-      </c>
-      <c r="D105" t="s">
-        <v>13</v>
-      </c>
-      <c r="E105" t="s">
-        <v>13</v>
-      </c>
-      <c r="F105" t="s">
+      <c r="G105" t="s">
+        <v>15</v>
+      </c>
+      <c r="H105" t="s">
         <v>609</v>
-      </c>
-      <c r="G105" t="s">
-        <v>15</v>
-      </c>
-      <c r="H105" t="s">
-        <v>545</v>
       </c>
       <c r="I105" t="s">
         <v>610</v>
@@ -6110,7 +6125,7 @@
         <v>613</v>
       </c>
       <c r="B106" t="s">
-        <v>543</v>
+        <v>548</v>
       </c>
       <c r="C106" t="s">
         <v>13</v>
@@ -6128,7 +6143,7 @@
         <v>15</v>
       </c>
       <c r="H106" t="s">
-        <v>323</v>
+        <v>550</v>
       </c>
       <c r="I106" t="s">
         <v>615</v>
@@ -6145,7 +6160,7 @@
         <v>618</v>
       </c>
       <c r="B107" t="s">
-        <v>537</v>
+        <v>548</v>
       </c>
       <c r="C107" t="s">
         <v>13</v>
@@ -6163,7 +6178,7 @@
         <v>15</v>
       </c>
       <c r="H107" t="s">
-        <v>604</v>
+        <v>328</v>
       </c>
       <c r="I107" t="s">
         <v>620</v>
@@ -6180,7 +6195,7 @@
         <v>623</v>
       </c>
       <c r="B108" t="s">
-        <v>104</v>
+        <v>542</v>
       </c>
       <c r="C108" t="s">
         <v>13</v>
@@ -6198,7 +6213,7 @@
         <v>15</v>
       </c>
       <c r="H108" t="s">
-        <v>379</v>
+        <v>609</v>
       </c>
       <c r="I108" t="s">
         <v>625</v>
@@ -6215,7 +6230,7 @@
         <v>628</v>
       </c>
       <c r="B109" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="C109" t="s">
         <v>13</v>
@@ -6233,7 +6248,7 @@
         <v>15</v>
       </c>
       <c r="H109" t="s">
-        <v>379</v>
+        <v>384</v>
       </c>
       <c r="I109" t="s">
         <v>630</v>
@@ -6250,7 +6265,7 @@
         <v>633</v>
       </c>
       <c r="B110" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="C110" t="s">
         <v>13</v>
@@ -6268,7 +6283,7 @@
         <v>15</v>
       </c>
       <c r="H110" t="s">
-        <v>379</v>
+        <v>384</v>
       </c>
       <c r="I110" t="s">
         <v>635</v>
@@ -6285,7 +6300,7 @@
         <v>638</v>
       </c>
       <c r="B111" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="C111" t="s">
         <v>13</v>
@@ -6303,7 +6318,7 @@
         <v>15</v>
       </c>
       <c r="H111" t="s">
-        <v>379</v>
+        <v>384</v>
       </c>
       <c r="I111" t="s">
         <v>640</v>
@@ -6320,7 +6335,7 @@
         <v>643</v>
       </c>
       <c r="B112" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="C112" t="s">
         <v>13</v>
@@ -6338,7 +6353,7 @@
         <v>15</v>
       </c>
       <c r="H112" t="s">
-        <v>532</v>
+        <v>384</v>
       </c>
       <c r="I112" t="s">
         <v>645</v>
@@ -6355,7 +6370,7 @@
         <v>648</v>
       </c>
       <c r="B113" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="C113" t="s">
         <v>13</v>
@@ -6373,7 +6388,7 @@
         <v>15</v>
       </c>
       <c r="H113" t="s">
-        <v>379</v>
+        <v>537</v>
       </c>
       <c r="I113" t="s">
         <v>650</v>
@@ -6390,51 +6405,51 @@
         <v>653</v>
       </c>
       <c r="B114" t="s">
+        <v>109</v>
+      </c>
+      <c r="C114" t="s">
+        <v>13</v>
+      </c>
+      <c r="D114" t="s">
+        <v>13</v>
+      </c>
+      <c r="E114" t="s">
+        <v>13</v>
+      </c>
+      <c r="F114" t="s">
         <v>654</v>
       </c>
-      <c r="C114" t="s">
-        <v>406</v>
-      </c>
-      <c r="D114" t="s">
-        <v>13</v>
-      </c>
-      <c r="E114" t="s">
+      <c r="G114" t="s">
+        <v>15</v>
+      </c>
+      <c r="H114" t="s">
+        <v>384</v>
+      </c>
+      <c r="I114" t="s">
         <v>655</v>
       </c>
-      <c r="F114" t="s">
+      <c r="J114" t="s">
         <v>656</v>
       </c>
-      <c r="G114" t="s">
-        <v>15</v>
-      </c>
-      <c r="H114" t="s">
-        <v>422</v>
-      </c>
-      <c r="I114" t="s">
+      <c r="K114" t="s">
         <v>657</v>
-      </c>
-      <c r="J114" t="s">
-        <v>658</v>
-      </c>
-      <c r="K114" t="s">
-        <v>659</v>
       </c>
     </row>
     <row r="115" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
+        <v>658</v>
+      </c>
+      <c r="B115" t="s">
+        <v>659</v>
+      </c>
+      <c r="C115" t="s">
+        <v>411</v>
+      </c>
+      <c r="D115" t="s">
+        <v>13</v>
+      </c>
+      <c r="E115" t="s">
         <v>660</v>
-      </c>
-      <c r="B115" t="s">
-        <v>654</v>
-      </c>
-      <c r="C115" t="s">
-        <v>413</v>
-      </c>
-      <c r="D115" t="s">
-        <v>13</v>
-      </c>
-      <c r="E115" t="s">
-        <v>655</v>
       </c>
       <c r="F115" t="s">
         <v>661</v>
@@ -6443,7 +6458,7 @@
         <v>15</v>
       </c>
       <c r="H115" t="s">
-        <v>422</v>
+        <v>427</v>
       </c>
       <c r="I115" t="s">
         <v>662</v>
@@ -6460,34 +6475,69 @@
         <v>665</v>
       </c>
       <c r="B116" t="s">
+        <v>659</v>
+      </c>
+      <c r="C116" t="s">
+        <v>418</v>
+      </c>
+      <c r="D116" t="s">
+        <v>13</v>
+      </c>
+      <c r="E116" t="s">
+        <v>660</v>
+      </c>
+      <c r="F116" t="s">
         <v>666</v>
       </c>
-      <c r="C116" t="s">
+      <c r="G116" t="s">
+        <v>15</v>
+      </c>
+      <c r="H116" t="s">
+        <v>427</v>
+      </c>
+      <c r="I116" t="s">
         <v>667</v>
       </c>
-      <c r="D116" t="s">
-        <v>13</v>
-      </c>
-      <c r="E116" t="s">
+      <c r="J116" t="s">
         <v>668</v>
       </c>
-      <c r="F116" t="s">
+      <c r="K116" t="s">
         <v>669</v>
       </c>
-      <c r="G116" t="s">
-        <v>15</v>
-      </c>
-      <c r="H116" t="s">
-        <v>422</v>
-      </c>
-      <c r="I116" t="s">
+    </row>
+    <row r="117" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
         <v>670</v>
       </c>
-      <c r="J116" t="s">
+      <c r="B117" t="s">
         <v>671</v>
       </c>
-      <c r="K116" t="s">
+      <c r="C117" t="s">
         <v>672</v>
+      </c>
+      <c r="D117" t="s">
+        <v>13</v>
+      </c>
+      <c r="E117" t="s">
+        <v>673</v>
+      </c>
+      <c r="F117" t="s">
+        <v>674</v>
+      </c>
+      <c r="G117" t="s">
+        <v>15</v>
+      </c>
+      <c r="H117" t="s">
+        <v>427</v>
+      </c>
+      <c r="I117" t="s">
+        <v>675</v>
+      </c>
+      <c r="J117" t="s">
+        <v>676</v>
+      </c>
+      <c r="K117" t="s">
+        <v>677</v>
       </c>
     </row>
   </sheetData>

</xml_diff>